<commit_message>
S03 WIP: packet sets v0.1 + TX priority policy
- policy/tx_priority_and_arbitration_v0_1.md: P0-P3, coalesce_key, hybrid expired_counter, intra-priority by expired_counter DESC
- policy/packet_sets_v0_1.md: Node_Core_Tail v0.1 (pos_quality16), Node_Operational v0.1 (battery16/radio8/uptime10m_u8), Node_Informative v0.1 (+ role_id); eligibility; Discovery + CONFLICT HW/FW u16 (options 1/2)
- master table: new fields/containers (pos_quality16, fix_type, pos_accuracy_bucket, pos_flags_small, pos_sats alias, battery16, radio8, uptime10m_u8, role_id, etc.); posFlags/sats marked superseded/alias; regenerated XLSX + CSV

Refs #351, #352

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
+++ b/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2285,7 +2285,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>posFlags</t>
+          <t>sats</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>pos_flags</t>
+          <t>sats</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>bit0=position valid; 1-7 reserved</t>
+          <t>satellite count; 0=not present</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2404,14 +2404,14 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>Position quality; does not revoke Core.</t>
+          <t>v0 canon. In v0.1 packed in pos_quality16; canonical field_key sats.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>uptimeSec</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>uptime_sec</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2468,17 +2468,17 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Node_Core_Tail</t>
+          <t>Node_Operational</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>tail1_packet_encoding_v0 §3.2</t>
+          <t>tail2_packet_encoding_v0 §3.2</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2488,12 +2488,12 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u32</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>satellite count; 0=not present</t>
+          <t>seconds; 0xFFFFFFFF=not present</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -2503,12 +2503,12 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>4294967295</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>32</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -2518,32 +2518,36 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Every Tail-1</t>
+          <t>on change + at forced Core</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>periodic</t>
+          <t>periodic+threshold</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>field_cadence: Tier B; packet is Node_Operational (0x04).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>uptimeSec</t>
+          <t>localAlias</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>LocalOnly</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2553,19 +2557,15 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>AppLocal</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>uptime_sec</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>in NodeEntry</t>
+          <t>app local storage</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2585,109 +2585,77 @@
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Node_Operational</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
-          <t>tail2_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>u32</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>seconds; 0xFFFFFFFF=not present</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>4294967295</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>on change + at forced Core</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>field_cadence: Tier B; packet is Node_Operational (0x04).</t>
+          <t>User-defined on phone; not over radio.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>localAlias</t>
+          <t>pos_age_s</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LocalOnly</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>CodeNow</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AppLocal</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>pos_age_s</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2695,16 +2663,24 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>app local storage</t>
+          <t>BLE snapshot</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
           <t>N</t>
@@ -2713,23 +2689,39 @@
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>Tail-1 pos quality; not in Core</t>
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>65535</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>B Tail-1</t>
         </is>
       </c>
       <c r="X20" t="inlineStr"/>
@@ -2738,14 +2730,14 @@
       <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>User-defined on phone; not over radio.</t>
+          <t>Domain; not in BeaconCore payload (position_quality_v0).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>pos_age_s</t>
+          <t>pos_valid</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2775,7 +2767,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>pos_age_s</t>
+          <t>pos_valid</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2785,7 +2777,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>BLE snapshot (flags bit1)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2795,12 +2787,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2809,41 +2801,29 @@
         </is>
       </c>
       <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Tail-1 pos quality; not in Core</t>
-        </is>
-      </c>
+      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>seconds</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>65535</t>
-        </is>
-      </c>
+          <t>flags bit 0x02; Core implies valid</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
+          <t>A Core</t>
         </is>
       </c>
       <c r="X21" t="inlineStr"/>
@@ -2852,24 +2832,24 @@
       <c r="AA21" t="inlineStr"/>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>Domain; not in BeaconCore payload (position_quality_v0).</t>
+          <t>Domain/BLE only; not on-air in BeaconCore (Core only when fix valid).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>pos_valid</t>
+          <t>is_grey</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2879,27 +2859,23 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>pos_valid</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>BLE snapshot (flags bit1)</t>
+          <t>computed at export</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2923,7 +2899,11 @@
         </is>
       </c>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>activity_state_v0</t>
+        </is>
+      </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
@@ -2933,7 +2913,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>flags bit 0x02; Core implies valid</t>
+          <t>flags bit 0x04; age_s &gt; expected_interval_s + grace_s</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -2945,23 +2925,19 @@
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>A Core</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr">
-        <is>
-          <t>Domain/BLE only; not on-air in BeaconCore (Core only when fix valid).</t>
-        </is>
-      </c>
+      <c r="AB22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>is_grey</t>
+          <t>last_seen_age_s</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2997,7 +2973,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>computed at export</t>
+          <t>computed at export from last_seen_ms</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -3007,12 +2983,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3021,30 +2997,22 @@
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>activity_state_v0</t>
-        </is>
-      </c>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>flags bit 0x04; age_s &gt; expected_interval_s + grace_s</t>
+          <t>(now_ms - last_seen_ms)/1000</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3054,22 +3022,26 @@
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="inlineStr"/>
-      <c r="AB23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>Derived for BLE; used for activity/grey.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>last_seen_age_s</t>
+          <t>in_use</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>LocalOnly</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3079,15 +3051,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>AppLocal</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>in_use</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>N</t>
@@ -3095,24 +3071,16 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>computed at export from last_seen_ms</t>
+          <t>internal slot only</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>N</t>
@@ -3124,14 +3092,10 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>u16</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>(now_ms - last_seen_ms)/1000</t>
-        </is>
-      </c>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr"/>
@@ -3146,14 +3110,14 @@
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>Derived for BLE; used for activity/grey.</t>
+          <t>Internal; not in BLE.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>in_use</t>
+          <t>is_self</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3183,26 +3147,34 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>in_use</t>
+          <t>is_self</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>internal slot only</t>
+          <t>BLE snapshot (flags bit0)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>N</t>
@@ -3217,10 +3189,18 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>flags bit 0x01</t>
+        </is>
+      </c>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W25" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3230,16 +3210,12 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr">
-        <is>
-          <t>Internal; not in BLE.</t>
-        </is>
-      </c>
+      <c r="AB25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>is_self</t>
+          <t>last_applied_tail_ref_core_seq16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3249,7 +3225,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LocalOnly</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3259,7 +3235,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>AppLocal</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3269,60 +3245,44 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>is_self</t>
+          <t>last_applied_tail_ref_core_seq16</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>BLE snapshot (flags bit0)</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>tail1_packet_encoding_v0; at most one Tail per Core</t>
+        </is>
+      </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>flags bit 0x01</t>
-        </is>
-      </c>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3332,12 +3292,16 @@
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="inlineStr"/>
-      <c r="AB26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>Variant 2: dedupe second Tail-1 for same ref_core_seq16.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>last_applied_tail_ref_core_seq16</t>
+          <t>short_id</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3347,7 +3311,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3357,7 +3321,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3367,33 +3331,41 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>last_applied_tail_ref_core_seq16</t>
+          <t>short_id</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>BLE snapshot</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>tail1_packet_encoding_v0; at most one Tail per Core</t>
-        </is>
-      </c>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
@@ -3401,10 +3373,18 @@
           <t>u16</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>CRC16-CCITT over node_id LE</t>
+        </is>
+      </c>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="W27" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3416,14 +3396,14 @@
       <c r="AA27" t="inlineStr"/>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>Variant 2: dedupe second Tail-1 for same ref_core_seq16.</t>
+          <t>Display only; not protocol key. Reserved 0x0000/0xFFFF handled.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>short_id</t>
+          <t>short_id_collision</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3453,7 +3433,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>short_id</t>
+          <t>short_id_collision</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3463,7 +3443,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>BLE snapshot (flags bit3)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -3473,12 +3453,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3492,19 +3472,19 @@
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>CRC16-CCITT over node_id LE</t>
+          <t>flags bit 0x08</t>
         </is>
       </c>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
@@ -3516,26 +3496,22 @@
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr"/>
-      <c r="AB28" t="inlineStr">
-        <is>
-          <t>Display only; not protocol key. Reserved 0x0000/0xFFFF handled.</t>
-        </is>
-      </c>
+      <c r="AB28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>short_id_collision</t>
+          <t>last_rx_rssi</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3545,7 +3521,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3555,7 +3531,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>short_id_collision</t>
+          <t>last_rx_rssi</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3565,7 +3541,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>BLE snapshot (flags bit3)</t>
+          <t>BLE snapshot</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3575,7 +3551,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>23</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -3589,24 +3565,28 @@
         </is>
       </c>
       <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>link_metrics_v0</t>
+        </is>
+      </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>i8</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>flags bit 0x08</t>
+          <t>dBm</t>
         </is>
       </c>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
@@ -3614,16 +3594,28 @@
           <t>Derived/Injected</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>on RX</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>event-driven</t>
+        </is>
+      </c>
       <c r="Z29" t="inlineStr"/>
       <c r="AA29" t="inlineStr"/>
-      <c r="AB29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>rssiLast; receiver-side only.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>last_rx_rssi</t>
+          <t>last_seen_ms</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3633,7 +3625,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3653,7 +3645,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>last_rx_rssi</t>
+          <t>last_seen_ms</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3663,54 +3655,38 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>internal; BLE exports last_seen_age_s derived</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>link_metrics_v0</t>
-        </is>
-      </c>
+      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>i8</t>
+          <t>u32</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>dBm</t>
+          <t>uptime ms</t>
         </is>
       </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+      <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3730,56 +3706,48 @@
       <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>rssiLast; receiver-side only.</t>
+          <t>Exported as lastSeenAgeS (age_s) in BLE.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>last_seen_ms</t>
+          <t>networkName</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CodeNow</t>
+          <t>Idea</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>last_seen_ms</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>internal; BLE exports last_seen_age_s derived</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>N</t>
@@ -3793,69 +3761,57 @@
         </is>
       </c>
       <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>index §4</t>
+        </is>
+      </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>u32</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>uptime ms</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>on RX</t>
-        </is>
-      </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>event-driven</t>
-        </is>
-      </c>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>Exported as lastSeenAgeS (age_s) in BLE.</t>
+          <t>NOT sent in v0 beacon; future session-join.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>networkName</t>
+          <t>hops</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Routing/Mesh</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3885,35 +3841,43 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
-          <t>index §4</t>
+          <t>meshtastic-nodetable.md §3</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>hops_away</t>
+        </is>
+      </c>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
       <c r="X32" t="inlineStr"/>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
       <c r="AA32" t="inlineStr"/>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>NOT sent in v0 beacon; future session-join.</t>
+          <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>hops</t>
+          <t>last_direct_time</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3923,7 +3887,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Routing/Mesh</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3963,21 +3927,17 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>meshtastic-nodetable.md §3</t>
+          <t>naviga_mesh_protocol_concept_v1_4.md</t>
         </is>
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>u8</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>hops_away</t>
-        </is>
-      </c>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
@@ -3992,14 +3952,14 @@
       <c r="AA33" t="inlineStr"/>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>No mesh routing in Naviga v0.</t>
+          <t>Time of last direct RX from this node; mesh concept. Non-goal v0.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>last_direct_time</t>
+          <t>next_hop</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4009,7 +3969,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Routing/Mesh</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4049,17 +4009,21 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr">
         <is>
-          <t>naviga_mesh_protocol_concept_v1_4.md</t>
+          <t>meshtastic-nodetable.md §3</t>
         </is>
       </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>last byte of node num</t>
+        </is>
+      </c>
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr"/>
@@ -4074,14 +4038,14 @@
       <c r="AA34" t="inlineStr"/>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>Time of last direct RX from this node; mesh concept. Non-goal v0.</t>
+          <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>next_hop</t>
+          <t>pos_history</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4091,7 +4055,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Routing/Mesh</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4101,7 +4065,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4131,19 +4095,19 @@
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr">
         <is>
-          <t>meshtastic-nodetable.md §3</t>
+          <t>naviga_mesh_protocol_concept_v1_4.md</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>array</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>last byte of node num</t>
+          <t>short history of positions</t>
         </is>
       </c>
       <c r="T35" t="inlineStr"/>
@@ -4160,14 +4124,14 @@
       <c r="AA35" t="inlineStr"/>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>No mesh routing in Naviga v0.</t>
+          <t>Optional pos_history_X; mesh concept. Non-goal v0.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>pos_history</t>
+          <t>role_params</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4177,7 +4141,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4224,12 +4188,12 @@
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>enum/params</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>short history of positions</t>
+          <t>role_pos_update_interval_X etc</t>
         </is>
       </c>
       <c r="T36" t="inlineStr"/>
@@ -4246,14 +4210,14 @@
       <c r="AA36" t="inlineStr"/>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>Optional pos_history_X; mesh concept. Non-goal v0.</t>
+          <t>Role-based delivery params; mesh concept. Non-goal v0.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>role_params</t>
+          <t>rssi_direct</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4263,7 +4227,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -4273,7 +4237,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4303,21 +4267,17 @@
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr">
         <is>
-          <t>naviga_mesh_protocol_concept_v1_4.md</t>
+          <t>meshtastic research</t>
         </is>
       </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>enum/params</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>role_pos_update_interval_X etc</t>
-        </is>
-      </c>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="inlineStr"/>
@@ -4332,14 +4292,14 @@
       <c r="AA37" t="inlineStr"/>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>Role-based delivery params; mesh concept. Non-goal v0.</t>
+          <t>Direct-link RSSI; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>rssi_direct</t>
+          <t>snr_direct</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4414,48 +4374,56 @@
       <c r="AA38" t="inlineStr"/>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>Direct-link RSSI; Mesh_future. Non-goal v0.</t>
+          <t>Direct-link SNR; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>snr_direct</t>
+          <t>posFlags</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>pos_flags</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>in NodeEntry</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr">
         <is>
           <t>N</t>
@@ -4465,38 +4433,1458 @@
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>meshtastic research</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
+          <t>tail1_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>bit0=position valid; 1-7 reserved</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr"/>
-      <c r="Y39" t="inlineStr"/>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>Direct-link SNR; Mesh_future. Non-goal v0.</t>
+          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>pos_sats</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>alias for sats</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr"/>
+      <c r="Y40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr"/>
+      <c r="AA40" t="inlineStr"/>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>Alias; superseded-by sats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>role_id</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Informative</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Node_Informative</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>role identifier</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr"/>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>periodic + changed-boost</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr"/>
+      <c r="AA41" t="inlineStr"/>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>battery16</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Telemetry/Health</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>pct7+charging1+eta10m8</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr"/>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
+      <c r="Z42" t="inlineStr"/>
+      <c r="AA42" t="inlineStr"/>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>v0.1 packed container.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>battery_pct7</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Telemetry/Health</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>7 bits in battery16; 0-100</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr"/>
+      <c r="Y43" t="inlineStr"/>
+      <c r="Z43" t="inlineStr"/>
+      <c r="AA43" t="inlineStr"/>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>Packed in battery16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>channel_throttle_step_u4</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>RadioContext</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>4 bits in radio8</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr"/>
+      <c r="Y44" t="inlineStr"/>
+      <c r="Z44" t="inlineStr"/>
+      <c r="AA44" t="inlineStr"/>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>Packed in radio8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>charging1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Telemetry/Health</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>1 bit in battery16</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr"/>
+      <c r="Y45" t="inlineStr"/>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>Packed in battery16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>eta10m8</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Telemetry/Health</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>8 bits in battery16; minutes to empty, 0=N/A</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr"/>
+      <c r="Y46" t="inlineStr"/>
+      <c r="Z46" t="inlineStr"/>
+      <c r="AA46" t="inlineStr"/>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>Packed in battery16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>fix_type</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>bits in pos_quality16: no_fix/2d/3d/reserved</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr"/>
+      <c r="Y47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr">
+        <is>
+          <t>Packed in pos_quality16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>pos_accuracy_bucket</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>bits in pos_quality16</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr"/>
+      <c r="Y48" t="inlineStr"/>
+      <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="inlineStr"/>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>Packed in pos_quality16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>pos_flags_small</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>bits in pos_quality16; supersedes posFlags in v0.1</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr"/>
+      <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>pos_quality16</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>packed: fix_type/sats/accuracy_bucket/pos_flags_small</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>radio8</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>RadioContext</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>txPower4+throttle4</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>v0.1 container.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>tx_power_step_u4</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>RadioContext</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>4 bits in radio8</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr"/>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr"/>
+      <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr"/>
+      <c r="AB52" t="inlineStr">
+        <is>
+          <t>Packed in radio8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>uptime10m_u8</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Telemetry/Health</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>uptime in 10-minute units; masked-for-compare</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr"/>
+      <c r="AA53" t="inlineStr"/>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>v0.1; eligibility snapshot mask.</t>
         </is>
       </c>
     </row>
@@ -4747,7 +6135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4933,46 +6321,70 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/packet_sets_v0_1.md</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
+          <t>Packet sets v0.1; Core_Tail/Operational/Informative payloads; CONFLICT HW/FW width.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
+          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>firmware/src/domain/node_table.cpp</t>
+          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>firmware/src/domain/node_table.cpp</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>firmware/src/domain/node_table.h</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>NodeEntry struct; NodeTable class; kRecordBytes=26.</t>
         </is>

</xml_diff>

<commit_message>
Add producer_status and source columns to master table
- Fields sheet: new columns producer_status (Implemented|Stubbed|Planned), source (HW|Derived|Injected|Config)
- Best-effort defaults from FIELD_DEFAULTS; every row has both values
- README: document columns as implementation-scope checklist
- Regenerated XLSX + fields_v0_1.csv (deterministic)

Refs #351, #352; dev umbrella #364.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
+++ b/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB53"/>
+  <dimension ref="A1:AD53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,6 +559,16 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>producer_status</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -669,6 +679,16 @@
           <t>Alive packet optional byte.</t>
         </is>
       </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Stubbed</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -795,6 +815,16 @@
           <t>Primary key; domain uint64 lower 48 bits.</t>
         </is>
       </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -913,6 +943,16 @@
           <t>Payload format version; first byte of payload.</t>
         </is>
       </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1039,6 +1079,16 @@
           <t>Core only with valid fix. BLE exports lat_e7 (i32).</t>
         </is>
       </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1165,6 +1215,16 @@
           <t>Core only with valid fix. BLE exports lon_e7 (i32).</t>
         </is>
       </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1283,6 +1343,16 @@
           <t>Back-reference to Core sample seq16; distinct from seq16 in Common.</t>
         </is>
       </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1415,6 +1485,16 @@
       <c r="AB8" t="inlineStr">
         <is>
           <t>Dedupe key (nodeId48, seq16). last_seq in NodeEntry.</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>HW</t>
         </is>
       </c>
     </row>
@@ -1503,6 +1583,16 @@
           <t>Derived; sent components posFlags, sats in Tail-1.</t>
         </is>
       </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1597,6 +1687,16 @@
         </is>
       </c>
       <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1711,6 +1811,16 @@
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1825,6 +1935,16 @@
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1949,6 +2069,16 @@
       <c r="AB13" t="inlineStr">
         <is>
           <t>Liveness hint; MUST NOT send on every Operational. Tier C.</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>Config</t>
         </is>
       </c>
     </row>
@@ -2053,6 +2183,16 @@
           <t>Canon name; firmware uses last_seen_ms.</t>
         </is>
       </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Injected</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2155,6 +2295,16 @@
           <t>Not in current BLE record.</t>
         </is>
       </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>Injected</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2281,6 +2431,16 @@
       </c>
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2407,6 +2567,16 @@
           <t>v0 canon. In v0.1 packed in pos_quality16; canonical field_key sats.</t>
         </is>
       </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2531,6 +2701,16 @@
       <c r="AB18" t="inlineStr">
         <is>
           <t>field_cadence: Tier B; packet is Node_Operational (0x04).</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>HW</t>
         </is>
       </c>
     </row>
@@ -2619,6 +2799,16 @@
           <t>User-defined on phone; not over radio.</t>
         </is>
       </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2733,6 +2923,16 @@
           <t>Domain; not in BeaconCore payload (position_quality_v0).</t>
         </is>
       </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2835,6 +3035,16 @@
           <t>Domain/BLE only; not on-air in BeaconCore (Core only when fix valid).</t>
         </is>
       </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2933,6 +3143,16 @@
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3027,6 +3247,16 @@
           <t>Derived for BLE; used for activity/grey.</t>
         </is>
       </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3113,6 +3343,16 @@
           <t>Internal; not in BLE.</t>
         </is>
       </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3211,6 +3451,16 @@
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr"/>
       <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3297,6 +3547,16 @@
           <t>Variant 2: dedupe second Tail-1 for same ref_core_seq16.</t>
         </is>
       </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3399,6 +3659,16 @@
           <t>Display only; not protocol key. Reserved 0x0000/0xFFFF handled.</t>
         </is>
       </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3497,6 +3767,16 @@
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr"/>
       <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3609,6 +3889,16 @@
       <c r="AB29" t="inlineStr">
         <is>
           <t>rssiLast; receiver-side only.</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>Injected</t>
         </is>
       </c>
     </row>
@@ -3707,6 +3997,16 @@
       <c r="AB30" t="inlineStr">
         <is>
           <t>Exported as lastSeenAgeS (age_s) in BLE.</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>Injected</t>
         </is>
       </c>
     </row>
@@ -3787,6 +4087,16 @@
           <t>NOT sent in v0 beacon; future session-join.</t>
         </is>
       </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3873,6 +4183,16 @@
           <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3955,6 +4275,16 @@
           <t>Time of last direct RX from this node; mesh concept. Non-goal v0.</t>
         </is>
       </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>Injected</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4041,6 +4371,16 @@
           <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4127,6 +4467,16 @@
           <t>Optional pos_history_X; mesh concept. Non-goal v0.</t>
         </is>
       </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4213,6 +4563,16 @@
           <t>Role-based delivery params; mesh concept. Non-goal v0.</t>
         </is>
       </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4295,6 +4655,16 @@
           <t>Direct-link RSSI; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>Injected</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4377,6 +4747,16 @@
           <t>Direct-link SNR; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>Injected</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4501,6 +4881,16 @@
       <c r="AB39" t="inlineStr">
         <is>
           <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>HW</t>
         </is>
       </c>
     </row>
@@ -4589,6 +4979,16 @@
           <t>Alias; superseded-by sats.</t>
         </is>
       </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4695,6 +5095,16 @@
           <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
         </is>
       </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4803,6 +5213,16 @@
       <c r="AB42" t="inlineStr">
         <is>
           <t>v0.1 packed container.</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>HW</t>
         </is>
       </c>
     </row>
@@ -4907,6 +5327,16 @@
           <t>Packed in battery16.</t>
         </is>
       </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5001,6 +5431,16 @@
           <t>Packed in radio8.</t>
         </is>
       </c>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5095,6 +5535,16 @@
           <t>Packed in battery16.</t>
         </is>
       </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5189,6 +5639,16 @@
           <t>Packed in battery16.</t>
         </is>
       </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5283,6 +5743,16 @@
           <t>Packed in pos_quality16.</t>
         </is>
       </c>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5377,6 +5847,16 @@
           <t>Packed in pos_quality16.</t>
         </is>
       </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5471,6 +5951,16 @@
           <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
         </is>
       </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5579,6 +6069,16 @@
       <c r="AB50" t="inlineStr">
         <is>
           <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>HW</t>
         </is>
       </c>
     </row>
@@ -5683,6 +6183,16 @@
           <t>v0.1 container.</t>
         </is>
       </c>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5777,6 +6287,16 @@
           <t>Packed in radio8.</t>
         </is>
       </c>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5885,6 +6405,16 @@
       <c r="AB53" t="inlineStr">
         <is>
           <t>v0.1; eligibility snapshot mask.</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>HW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S03 WIP: freeze Identity/Naming + Persistence/Eviction block
- Add canonical block doc: identity_naming_persistence_eviction_v0_1.md
  (is_self, node_id, short_id, short_id_collision, node_name, authority rule,
  persistence/eviction v1 scope, out-of-scope networkName & ownership)
- Link packet_sets_v0_1 and tx_priority_and_arbitration_v0_1 to block doc
- Master table: add node_name (Planned, Config); update networkName/localAlias
  notes; add block to sources; regenerate CSV + XLSX
- Issues: #367 (FW persistence v1 + eviction v1), #368 (FW/BLE self node_name),
  #369 (App local phone name + authoritative rule)

Refs #351 #352 #364.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
+++ b/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD53"/>
+  <dimension ref="A1:AD54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2796,7 +2796,7 @@
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>User-defined on phone; not over radio.</t>
+          <t>Local phone name; fallback when node_name (authoritative) empty. User-defined on phone; not over radio. Replaced by node-reported node_name when present (authority rule).</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -4084,7 +4084,7 @@
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>NOT sent in v0 beacon; future session-join.</t>
+          <t>Out-of-scope S03; NOT sent in v0 beacon; future session-join.</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -6415,6 +6415,102 @@
       <c r="AD53" t="inlineStr">
         <is>
           <t>HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>node_name</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>self-only in NVS (S03); not on-air in S03</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>identity_naming_persistence_eviction_v0_1</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr"/>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr"/>
+      <c r="Y54" t="inlineStr"/>
+      <c r="Z54" t="inlineStr"/>
+      <c r="AA54" t="inlineStr"/>
+      <c r="AB54" t="inlineStr">
+        <is>
+          <t>Human-readable name. S03: self set via BLE, persisted NVS; remote usually empty. Sxx: remote from over-air; authority rule: node-reported replaces local. UI: node_name -&gt; local phone name -&gt; short_id.</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>Config</t>
         </is>
       </c>
     </row>
@@ -6665,7 +6761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6851,70 +6947,82 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/policy/packet_sets_v0_1.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/identity_naming_persistence_eviction_v0_1.md</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Packet sets v0.1; Core_Tail/Operational/Informative payloads; CONFLICT HW/FW width.</t>
+          <t>S03 block: Identity, naming (node_name, authority rule), persistence/eviction scope; out-of-scope networkName, ownership.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/packet_sets_v0_1.md</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
+          <t>Packet sets v0.1; Core_Tail/Operational/Informative payloads; CONFLICT HW/FW width.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
+          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
+          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
+          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>firmware/src/domain/node_table.cpp</t>
+          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>firmware/src/domain/node_table.cpp</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>firmware/src/domain/node_table.h</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>NodeEntry struct; NodeTable class; kRecordBytes=26.</t>
         </is>

</xml_diff>

<commit_message>
S03 WIP: freeze Identity/Naming + Persistence/Eviction block (#370)
- Add canonical block doc: identity_naming_persistence_eviction_v0_1.md
  (is_self, node_id, short_id, short_id_collision, node_name, authority rule,
  persistence/eviction v1 scope, out-of-scope networkName & ownership)
- Link packet_sets_v0_1 and tx_priority_and_arbitration_v0_1 to block doc
- Master table: add node_name (Planned, Config); update networkName/localAlias
  notes; add block to sources; regenerate CSV + XLSX
- Issues: #367 (FW persistence v1 + eviction v1), #368 (FW/BLE self node_name),
  #369 (App local phone name + authoritative rule)

Refs #351 #352 #364.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
+++ b/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD53"/>
+  <dimension ref="A1:AD54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2796,7 +2796,7 @@
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>User-defined on phone; not over radio.</t>
+          <t>Local phone name; fallback when node_name (authoritative) empty. User-defined on phone; not over radio. Replaced by node-reported node_name when present (authority rule).</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -4084,7 +4084,7 @@
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>NOT sent in v0 beacon; future session-join.</t>
+          <t>Out-of-scope S03; NOT sent in v0 beacon; future session-join.</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -6415,6 +6415,102 @@
       <c r="AD53" t="inlineStr">
         <is>
           <t>HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>node_name</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>self-only in NVS (S03); not on-air in S03</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>identity_naming_persistence_eviction_v0_1</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr"/>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr"/>
+      <c r="Y54" t="inlineStr"/>
+      <c r="Z54" t="inlineStr"/>
+      <c r="AA54" t="inlineStr"/>
+      <c r="AB54" t="inlineStr">
+        <is>
+          <t>Human-readable name. S03: self set via BLE, persisted NVS; remote usually empty. Sxx: remote from over-air; authority rule: node-reported replaces local. UI: node_name -&gt; local phone name -&gt; short_id.</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>Config</t>
         </is>
       </c>
     </row>
@@ -6665,7 +6761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6851,70 +6947,82 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/policy/packet_sets_v0_1.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/identity_naming_persistence_eviction_v0_1.md</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Packet sets v0.1; Core_Tail/Operational/Informative payloads; CONFLICT HW/FW width.</t>
+          <t>S03 block: Identity, naming (node_name, authority rule), persistence/eviction scope; out-of-scope networkName, ownership.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/packet_sets_v0_1.md</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
+          <t>Packet sets v0.1; Core_Tail/Operational/Informative payloads; CONFLICT HW/FW width.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
+          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
+          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
+          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>firmware/src/domain/node_table.cpp</t>
+          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>firmware/src/domain/node_table.cpp</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>firmware/src/domain/node_table.h</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>NodeEntry struct; NodeTable class; kRecordBytes=26.</t>
         </is>

</xml_diff>

<commit_message>
S03 WIP: presence semantics + rename is_stale
- Add presence_and_age_semantics_v0_1.md: S03 minimal presence/age model
  (last_seen_ms, last_seen_age_s, is_stale, pos_age_s; expected_interval_s =
  max_silence_10s*10; grace_s TBD; self TX presence special-case)
- Master table: is_stale (Implemented, Derived) + is_grey as Superseded alias;
  notes for expected_interval_s, self TX presence; last_seen_age_s/pos_age_s
  as S03 minimal; add presence doc to sources
- Regenerate XLSX + CSV

Refs #351 #352 #371 #372.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
+++ b/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD54"/>
+  <dimension ref="A1:AD55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2920,7 +2920,7 @@
       <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>Domain; not in BeaconCore payload (position_quality_v0).</t>
+          <t>S03 minimal. Age of last known position sample (independent from presence). Domain; not in BeaconCore payload (position_quality_v0).</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -3049,7 +3049,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>is_grey</t>
+          <t>is_stale</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3111,7 +3111,7 @@
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
-          <t>activity_state_v0</t>
+          <t>presence_and_age_semantics_v0_1</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -3123,7 +3123,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>flags bit 0x04; age_s &gt; expected_interval_s + grace_s</t>
+          <t>flags bit 0x04; last_seen_age_s &gt; expected_interval_s + grace_s</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3142,7 +3142,11 @@
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>S03 minimal. expected_interval_s = max_silence_10s * 10; grace_s hysteresis TBD. Self: TX heartbeat updates last_seen_ms so self does not appear stale (presence_and_age_semantics_v0_1).</t>
+        </is>
+      </c>
       <c r="AC22" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3244,7 +3248,7 @@
       <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>Derived for BLE; used for activity/grey.</t>
+          <t>S03 minimal. floor((now_ms - last_seen_ms)/1000) at export; BLE convenience; derived from last_seen_ms. See presence_and_age_semantics_v0_1.</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -4761,17 +4765,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>posFlags</t>
+          <t>is_grey</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4781,106 +4785,74 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>pos_flags</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>in NodeEntry</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Node_Core_Tail</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>tail1_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>same as is_stale (flags bit 0x04)</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>u8</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>bit0=position valid; 1-7 reserved</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
+          <t>Alias; superseded-by is_stale (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
@@ -4890,14 +4862,14 @@
       </c>
       <c r="AD39" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>pos_sats</t>
+          <t>posFlags</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4922,16 +4894,24 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>pos_flags</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>in NodeEntry</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr">
         <is>
           <t>N</t>
@@ -4941,17 +4921,29 @@
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>packet_sets_v0_1</t>
-        </is>
-      </c>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
+          <t>tail1_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R40" t="inlineStr">
         <is>
           <t>u8</t>
@@ -4959,56 +4951,76 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>alias for sats</t>
-        </is>
-      </c>
-      <c r="T40" t="inlineStr"/>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr"/>
+          <t>bit0=position valid; 1-7 reserved</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W40" t="inlineStr">
         <is>
           <t>B Tail-1</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr"/>
-      <c r="Y40" t="inlineStr"/>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z40" t="inlineStr"/>
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>Alias; superseded-by sats.</t>
+          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
         </is>
       </c>
       <c r="AC40" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD40" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>role_id</t>
+          <t>pos_sats</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>WIP</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -5037,25 +5049,17 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>Node_Informative</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
           <t>packet_sets_v0_1</t>
         </is>
       </c>
       <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
           <t>u8</t>
@@ -5063,36 +5067,24 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>role identifier</t>
+          <t>alias for sats</t>
         </is>
       </c>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
+      <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
-        </is>
-      </c>
-      <c r="X41" t="inlineStr">
-        <is>
-          <t>periodic + changed-boost</t>
-        </is>
-      </c>
-      <c r="Y41" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr"/>
+      <c r="Y41" t="inlineStr"/>
       <c r="Z41" t="inlineStr"/>
       <c r="AA41" t="inlineStr"/>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
+          <t>Alias; superseded-by sats.</t>
         </is>
       </c>
       <c r="AC41" t="inlineStr">
@@ -5102,24 +5094,24 @@
       </c>
       <c r="AD41" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>battery16</t>
+          <t>role_id</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5158,7 +5150,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Node_Operational</t>
+          <t>Node_Informative</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -5166,11 +5158,7 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr">
         <is>
           <t>OPT</t>
@@ -5178,19 +5166,19 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>pct7+charging1+eta10m8</t>
+          <t>role identifier</t>
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>TODO</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
@@ -5200,19 +5188,19 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>on change + min_interval</t>
+          <t>periodic + changed-boost</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>periodic+threshold</t>
+          <t>periodic</t>
         </is>
       </c>
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>v0.1 packed container.</t>
+          <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
         </is>
       </c>
       <c r="AC42" t="inlineStr">
@@ -5222,14 +5210,14 @@
       </c>
       <c r="AD42" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>battery_pct7</t>
+          <t>battery16</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5286,31 +5274,31 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>7 bits in battery16; 0-100</t>
-        </is>
-      </c>
-      <c r="T43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+          <t>pct7+charging1+eta10m8</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
@@ -5318,13 +5306,21 @@
           <t>C Tail-2</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr"/>
-      <c r="Y43" t="inlineStr"/>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
       <c r="Z43" t="inlineStr"/>
       <c r="AA43" t="inlineStr"/>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>Packed in battery16.</t>
+          <t>v0.1 packed container.</t>
         </is>
       </c>
       <c r="AC43" t="inlineStr">
@@ -5341,7 +5337,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>channel_throttle_step_u4</t>
+          <t>battery_pct7</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5351,7 +5347,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5407,14 +5403,22 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>4 bits in radio8</t>
-        </is>
-      </c>
-      <c r="T44" t="inlineStr"/>
-      <c r="U44" t="inlineStr"/>
+          <t>7 bits in battery16; 0-100</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
@@ -5428,7 +5432,7 @@
       <c r="AA44" t="inlineStr"/>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>Packed in radio8.</t>
+          <t>Packed in battery16.</t>
         </is>
       </c>
       <c r="AC44" t="inlineStr">
@@ -5438,14 +5442,14 @@
       </c>
       <c r="AD44" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>charging1</t>
+          <t>channel_throttle_step_u4</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5455,7 +5459,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5506,19 +5510,19 @@
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>1 bit in battery16</t>
+          <t>4 bits in radio8</t>
         </is>
       </c>
       <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
@@ -5532,7 +5536,7 @@
       <c r="AA45" t="inlineStr"/>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>Packed in battery16.</t>
+          <t>Packed in radio8.</t>
         </is>
       </c>
       <c r="AC45" t="inlineStr">
@@ -5542,14 +5546,14 @@
       </c>
       <c r="AD45" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>eta10m8</t>
+          <t>charging1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5610,19 +5614,19 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>8 bits in battery16; minutes to empty, 0=N/A</t>
+          <t>1 bit in battery16</t>
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
@@ -5646,14 +5650,14 @@
       </c>
       <c r="AD46" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>fix_type</t>
+          <t>eta10m8</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5663,7 +5667,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5702,7 +5706,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Node_Core_Tail</t>
+          <t>Node_Operational</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -5714,24 +5718,24 @@
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>bits in pos_quality16: no_fix/2d/3d/reserved</t>
+          <t>8 bits in battery16; minutes to empty, 0=N/A</t>
         </is>
       </c>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X47" t="inlineStr"/>
@@ -5740,7 +5744,7 @@
       <c r="AA47" t="inlineStr"/>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>Packed in pos_quality16.</t>
+          <t>Packed in battery16.</t>
         </is>
       </c>
       <c r="AC47" t="inlineStr">
@@ -5750,14 +5754,14 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>pos_accuracy_bucket</t>
+          <t>fix_type</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5818,19 +5822,19 @@
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>bits in pos_quality16</t>
+          <t>bits in pos_quality16: no_fix/2d/3d/reserved</t>
         </is>
       </c>
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W48" t="inlineStr">
@@ -5854,14 +5858,14 @@
       </c>
       <c r="AD48" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>pos_flags_small</t>
+          <t>pos_accuracy_bucket</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5927,14 +5931,14 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>bits in pos_quality16; supersedes posFlags in v0.1</t>
+          <t>bits in pos_quality16</t>
         </is>
       </c>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="W49" t="inlineStr">
@@ -5948,7 +5952,7 @@
       <c r="AA49" t="inlineStr"/>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
+          <t>Packed in pos_quality16.</t>
         </is>
       </c>
       <c r="AC49" t="inlineStr">
@@ -5958,14 +5962,14 @@
       </c>
       <c r="AD49" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>pos_quality16</t>
+          <t>pos_flags_small</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -6022,31 +6026,23 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>packed: fix_type/sats/accuracy_bucket/pos_flags_small</t>
+          <t>bits in pos_quality16; supersedes posFlags in v0.1</t>
         </is>
       </c>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>5</t>
         </is>
       </c>
       <c r="W50" t="inlineStr">
@@ -6054,21 +6050,13 @@
           <t>B Tail-1</t>
         </is>
       </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y50" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
       <c r="Z50" t="inlineStr"/>
       <c r="AA50" t="inlineStr"/>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
+          <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
         </is>
       </c>
       <c r="AC50" t="inlineStr">
@@ -6085,7 +6073,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>radio8</t>
+          <t>pos_quality16</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -6095,7 +6083,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6134,7 +6122,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>Node_Operational</t>
+          <t>Node_Core_Tail</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -6144,7 +6132,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -6154,33 +6142,41 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>txPower4+throttle4</t>
+          <t>packed: fix_type/sats/accuracy_bucket/pos_flags_small</t>
         </is>
       </c>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
-        </is>
-      </c>
-      <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr"/>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z51" t="inlineStr"/>
       <c r="AA51" t="inlineStr"/>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>v0.1 container.</t>
+          <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
         </is>
       </c>
       <c r="AC51" t="inlineStr">
@@ -6197,7 +6193,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>tx_power_step_u4</t>
+          <t>radio8</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6254,8 +6250,16 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R52" t="inlineStr">
         <is>
           <t>u8</t>
@@ -6263,14 +6267,14 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>4 bits in radio8</t>
+          <t>txPower4+throttle4</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
       <c r="V52" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W52" t="inlineStr">
@@ -6284,7 +6288,7 @@
       <c r="AA52" t="inlineStr"/>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>Packed in radio8.</t>
+          <t>v0.1 container.</t>
         </is>
       </c>
       <c r="AC52" t="inlineStr">
@@ -6301,7 +6305,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>uptime10m_u8</t>
+          <t>tx_power_step_u4</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6311,7 +6315,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6358,16 +6362,8 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
           <t>u8</t>
@@ -6375,14 +6371,14 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>uptime in 10-minute units; masked-for-compare</t>
+          <t>4 bits in radio8</t>
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W53" t="inlineStr">
@@ -6390,21 +6386,13 @@
           <t>C Tail-2</t>
         </is>
       </c>
-      <c r="X53" t="inlineStr">
-        <is>
-          <t>on change + min_interval</t>
-        </is>
-      </c>
-      <c r="Y53" t="inlineStr">
-        <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
+      <c r="X53" t="inlineStr"/>
+      <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr"/>
       <c r="AA53" t="inlineStr"/>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>v0.1; eligibility snapshot mask.</t>
+          <t>Packed in radio8.</t>
         </is>
       </c>
       <c r="AC53" t="inlineStr">
@@ -6421,17 +6409,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>node_name</t>
+          <t>uptime10m_u8</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6452,63 +6440,183 @@
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>self-only in NVS (S03); not on-air in S03</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>identity_naming_persistence_eviction_v0_1</t>
-        </is>
-      </c>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S54" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>uptime in 10-minute units; masked-for-compare</t>
+        </is>
+      </c>
       <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr"/>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X54" t="inlineStr"/>
-      <c r="Y54" t="inlineStr"/>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="inlineStr"/>
       <c r="AB54" t="inlineStr">
         <is>
+          <t>v0.1; eligibility snapshot mask.</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>node_name</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>self-only in NVS (S03); not on-air in S03</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>identity_naming_persistence_eviction_v0_1</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr"/>
+      <c r="Y55" t="inlineStr"/>
+      <c r="Z55" t="inlineStr"/>
+      <c r="AA55" t="inlineStr"/>
+      <c r="AB55" t="inlineStr">
+        <is>
           <t>Human-readable name. S03: self set via BLE, persisted NVS; remote usually empty. Sxx: remote from over-air; authority rule: node-reported replaces local. UI: node_name -&gt; local phone name -&gt; short_id.</t>
         </is>
       </c>
-      <c r="AC54" t="inlineStr">
+      <c r="AC55" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="AD54" t="inlineStr">
+      <c r="AD55" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
@@ -6761,7 +6869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6971,58 +7079,70 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/presence_and_age_semantics_v0_1.md</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
+          <t>S03 minimal presence/age: last_seen_ms, last_seen_age_s, is_stale (rename from is_grey), pos_age_s; expected_interval_s=max_silence_10s*10; grace_s TBD; self TX presence.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
+          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
+          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
+          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>firmware/src/domain/node_table.cpp</t>
+          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>firmware/src/domain/node_table.cpp</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>firmware/src/domain/node_table.h</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>NodeEntry struct; NodeTable class; kRecordBytes=26.</t>
         </is>

</xml_diff>

<commit_message>
S03 WIP: presence semantics + rename is_stale (#373)
- Add presence_and_age_semantics_v0_1.md: S03 minimal presence/age model
  (last_seen_ms, last_seen_age_s, is_stale, pos_age_s; expected_interval_s =
  max_silence_10s*10; grace_s TBD; self TX presence special-case)
- Master table: is_stale (Implemented, Derived) + is_grey as Superseded alias;
  notes for expected_interval_s, self TX presence; last_seen_age_s/pos_age_s
  as S03 minimal; add presence doc to sources
- Regenerate XLSX + CSV

Refs #351 #352 #371 #372.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
+++ b/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD54"/>
+  <dimension ref="A1:AD55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2920,7 +2920,7 @@
       <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>Domain; not in BeaconCore payload (position_quality_v0).</t>
+          <t>S03 minimal. Age of last known position sample (independent from presence). Domain; not in BeaconCore payload (position_quality_v0).</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -3049,7 +3049,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>is_grey</t>
+          <t>is_stale</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3111,7 +3111,7 @@
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
-          <t>activity_state_v0</t>
+          <t>presence_and_age_semantics_v0_1</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -3123,7 +3123,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>flags bit 0x04; age_s &gt; expected_interval_s + grace_s</t>
+          <t>flags bit 0x04; last_seen_age_s &gt; expected_interval_s + grace_s</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3142,7 +3142,11 @@
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>S03 minimal. expected_interval_s = max_silence_10s * 10; grace_s hysteresis TBD. Self: TX heartbeat updates last_seen_ms so self does not appear stale (presence_and_age_semantics_v0_1).</t>
+        </is>
+      </c>
       <c r="AC22" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3244,7 +3248,7 @@
       <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>Derived for BLE; used for activity/grey.</t>
+          <t>S03 minimal. floor((now_ms - last_seen_ms)/1000) at export; BLE convenience; derived from last_seen_ms. See presence_and_age_semantics_v0_1.</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -4761,17 +4765,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>posFlags</t>
+          <t>is_grey</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4781,106 +4785,74 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>pos_flags</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>in NodeEntry</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Node_Core_Tail</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>tail1_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>same as is_stale (flags bit 0x04)</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>u8</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>bit0=position valid; 1-7 reserved</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
+          <t>Alias; superseded-by is_stale (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
@@ -4890,14 +4862,14 @@
       </c>
       <c r="AD39" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>pos_sats</t>
+          <t>posFlags</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4922,16 +4894,24 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>pos_flags</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>in NodeEntry</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr">
         <is>
           <t>N</t>
@@ -4941,17 +4921,29 @@
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>packet_sets_v0_1</t>
-        </is>
-      </c>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
+          <t>tail1_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R40" t="inlineStr">
         <is>
           <t>u8</t>
@@ -4959,56 +4951,76 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>alias for sats</t>
-        </is>
-      </c>
-      <c r="T40" t="inlineStr"/>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr"/>
+          <t>bit0=position valid; 1-7 reserved</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W40" t="inlineStr">
         <is>
           <t>B Tail-1</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr"/>
-      <c r="Y40" t="inlineStr"/>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z40" t="inlineStr"/>
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>Alias; superseded-by sats.</t>
+          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
         </is>
       </c>
       <c r="AC40" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD40" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>role_id</t>
+          <t>pos_sats</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>WIP</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -5037,25 +5049,17 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>Node_Informative</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
           <t>packet_sets_v0_1</t>
         </is>
       </c>
       <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
           <t>u8</t>
@@ -5063,36 +5067,24 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>role identifier</t>
+          <t>alias for sats</t>
         </is>
       </c>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
+      <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
-        </is>
-      </c>
-      <c r="X41" t="inlineStr">
-        <is>
-          <t>periodic + changed-boost</t>
-        </is>
-      </c>
-      <c r="Y41" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr"/>
+      <c r="Y41" t="inlineStr"/>
       <c r="Z41" t="inlineStr"/>
       <c r="AA41" t="inlineStr"/>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
+          <t>Alias; superseded-by sats.</t>
         </is>
       </c>
       <c r="AC41" t="inlineStr">
@@ -5102,24 +5094,24 @@
       </c>
       <c r="AD41" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>battery16</t>
+          <t>role_id</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5158,7 +5150,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Node_Operational</t>
+          <t>Node_Informative</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -5166,11 +5158,7 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr">
         <is>
           <t>OPT</t>
@@ -5178,19 +5166,19 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>pct7+charging1+eta10m8</t>
+          <t>role identifier</t>
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>TODO</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
@@ -5200,19 +5188,19 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>on change + min_interval</t>
+          <t>periodic + changed-boost</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>periodic+threshold</t>
+          <t>periodic</t>
         </is>
       </c>
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>v0.1 packed container.</t>
+          <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
         </is>
       </c>
       <c r="AC42" t="inlineStr">
@@ -5222,14 +5210,14 @@
       </c>
       <c r="AD42" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>battery_pct7</t>
+          <t>battery16</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5286,31 +5274,31 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>7 bits in battery16; 0-100</t>
-        </is>
-      </c>
-      <c r="T43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+          <t>pct7+charging1+eta10m8</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
@@ -5318,13 +5306,21 @@
           <t>C Tail-2</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr"/>
-      <c r="Y43" t="inlineStr"/>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
       <c r="Z43" t="inlineStr"/>
       <c r="AA43" t="inlineStr"/>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>Packed in battery16.</t>
+          <t>v0.1 packed container.</t>
         </is>
       </c>
       <c r="AC43" t="inlineStr">
@@ -5341,7 +5337,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>channel_throttle_step_u4</t>
+          <t>battery_pct7</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5351,7 +5347,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5407,14 +5403,22 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>4 bits in radio8</t>
-        </is>
-      </c>
-      <c r="T44" t="inlineStr"/>
-      <c r="U44" t="inlineStr"/>
+          <t>7 bits in battery16; 0-100</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
@@ -5428,7 +5432,7 @@
       <c r="AA44" t="inlineStr"/>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>Packed in radio8.</t>
+          <t>Packed in battery16.</t>
         </is>
       </c>
       <c r="AC44" t="inlineStr">
@@ -5438,14 +5442,14 @@
       </c>
       <c r="AD44" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>charging1</t>
+          <t>channel_throttle_step_u4</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5455,7 +5459,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5506,19 +5510,19 @@
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>1 bit in battery16</t>
+          <t>4 bits in radio8</t>
         </is>
       </c>
       <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
@@ -5532,7 +5536,7 @@
       <c r="AA45" t="inlineStr"/>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>Packed in battery16.</t>
+          <t>Packed in radio8.</t>
         </is>
       </c>
       <c r="AC45" t="inlineStr">
@@ -5542,14 +5546,14 @@
       </c>
       <c r="AD45" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>eta10m8</t>
+          <t>charging1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5610,19 +5614,19 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>8 bits in battery16; minutes to empty, 0=N/A</t>
+          <t>1 bit in battery16</t>
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
@@ -5646,14 +5650,14 @@
       </c>
       <c r="AD46" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>fix_type</t>
+          <t>eta10m8</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5663,7 +5667,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5702,7 +5706,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Node_Core_Tail</t>
+          <t>Node_Operational</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -5714,24 +5718,24 @@
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>bits in pos_quality16: no_fix/2d/3d/reserved</t>
+          <t>8 bits in battery16; minutes to empty, 0=N/A</t>
         </is>
       </c>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X47" t="inlineStr"/>
@@ -5740,7 +5744,7 @@
       <c r="AA47" t="inlineStr"/>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>Packed in pos_quality16.</t>
+          <t>Packed in battery16.</t>
         </is>
       </c>
       <c r="AC47" t="inlineStr">
@@ -5750,14 +5754,14 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>pos_accuracy_bucket</t>
+          <t>fix_type</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5818,19 +5822,19 @@
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>bits in pos_quality16</t>
+          <t>bits in pos_quality16: no_fix/2d/3d/reserved</t>
         </is>
       </c>
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W48" t="inlineStr">
@@ -5854,14 +5858,14 @@
       </c>
       <c r="AD48" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>pos_flags_small</t>
+          <t>pos_accuracy_bucket</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5927,14 +5931,14 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>bits in pos_quality16; supersedes posFlags in v0.1</t>
+          <t>bits in pos_quality16</t>
         </is>
       </c>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="W49" t="inlineStr">
@@ -5948,7 +5952,7 @@
       <c r="AA49" t="inlineStr"/>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
+          <t>Packed in pos_quality16.</t>
         </is>
       </c>
       <c r="AC49" t="inlineStr">
@@ -5958,14 +5962,14 @@
       </c>
       <c r="AD49" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>pos_quality16</t>
+          <t>pos_flags_small</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -6022,31 +6026,23 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>packed: fix_type/sats/accuracy_bucket/pos_flags_small</t>
+          <t>bits in pos_quality16; supersedes posFlags in v0.1</t>
         </is>
       </c>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>5</t>
         </is>
       </c>
       <c r="W50" t="inlineStr">
@@ -6054,21 +6050,13 @@
           <t>B Tail-1</t>
         </is>
       </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y50" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
       <c r="Z50" t="inlineStr"/>
       <c r="AA50" t="inlineStr"/>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
+          <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
         </is>
       </c>
       <c r="AC50" t="inlineStr">
@@ -6085,7 +6073,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>radio8</t>
+          <t>pos_quality16</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -6095,7 +6083,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6134,7 +6122,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>Node_Operational</t>
+          <t>Node_Core_Tail</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -6144,7 +6132,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -6154,33 +6142,41 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>txPower4+throttle4</t>
+          <t>packed: fix_type/sats/accuracy_bucket/pos_flags_small</t>
         </is>
       </c>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
-        </is>
-      </c>
-      <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr"/>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z51" t="inlineStr"/>
       <c r="AA51" t="inlineStr"/>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>v0.1 container.</t>
+          <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
         </is>
       </c>
       <c r="AC51" t="inlineStr">
@@ -6197,7 +6193,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>tx_power_step_u4</t>
+          <t>radio8</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6254,8 +6250,16 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R52" t="inlineStr">
         <is>
           <t>u8</t>
@@ -6263,14 +6267,14 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>4 bits in radio8</t>
+          <t>txPower4+throttle4</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
       <c r="V52" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W52" t="inlineStr">
@@ -6284,7 +6288,7 @@
       <c r="AA52" t="inlineStr"/>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>Packed in radio8.</t>
+          <t>v0.1 container.</t>
         </is>
       </c>
       <c r="AC52" t="inlineStr">
@@ -6301,7 +6305,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>uptime10m_u8</t>
+          <t>tx_power_step_u4</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6311,7 +6315,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6358,16 +6362,8 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
           <t>u8</t>
@@ -6375,14 +6371,14 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>uptime in 10-minute units; masked-for-compare</t>
+          <t>4 bits in radio8</t>
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W53" t="inlineStr">
@@ -6390,21 +6386,13 @@
           <t>C Tail-2</t>
         </is>
       </c>
-      <c r="X53" t="inlineStr">
-        <is>
-          <t>on change + min_interval</t>
-        </is>
-      </c>
-      <c r="Y53" t="inlineStr">
-        <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
+      <c r="X53" t="inlineStr"/>
+      <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr"/>
       <c r="AA53" t="inlineStr"/>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>v0.1; eligibility snapshot mask.</t>
+          <t>Packed in radio8.</t>
         </is>
       </c>
       <c r="AC53" t="inlineStr">
@@ -6421,17 +6409,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>node_name</t>
+          <t>uptime10m_u8</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6452,63 +6440,183 @@
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>self-only in NVS (S03); not on-air in S03</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>identity_naming_persistence_eviction_v0_1</t>
-        </is>
-      </c>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S54" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>uptime in 10-minute units; masked-for-compare</t>
+        </is>
+      </c>
       <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr"/>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X54" t="inlineStr"/>
-      <c r="Y54" t="inlineStr"/>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="inlineStr"/>
       <c r="AB54" t="inlineStr">
         <is>
+          <t>v0.1; eligibility snapshot mask.</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>node_name</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>self-only in NVS (S03); not on-air in S03</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>identity_naming_persistence_eviction_v0_1</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr"/>
+      <c r="Y55" t="inlineStr"/>
+      <c r="Z55" t="inlineStr"/>
+      <c r="AA55" t="inlineStr"/>
+      <c r="AB55" t="inlineStr">
+        <is>
           <t>Human-readable name. S03: self set via BLE, persisted NVS; remote usually empty. Sxx: remote from over-air; authority rule: node-reported replaces local. UI: node_name -&gt; local phone name -&gt; short_id.</t>
         </is>
       </c>
-      <c r="AC54" t="inlineStr">
+      <c r="AC55" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="AD54" t="inlineStr">
+      <c r="AD55" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
@@ -6761,7 +6869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6971,58 +7079,70 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/presence_and_age_semantics_v0_1.md</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
+          <t>S03 minimal presence/age: last_seen_ms, last_seen_age_s, is_stale (rename from is_grey), pos_age_s; expected_interval_s=max_silence_10s*10; grace_s TBD; self TX presence.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
+          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
+          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
+          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>firmware/src/domain/node_table.cpp</t>
+          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>firmware/src/domain/node_table.cpp</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>firmware/src/domain/node_table.h</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>NodeEntry struct; NodeTable class; kRecordBytes=26.</t>
         </is>

</xml_diff>

<commit_message>
S03: Record decision — aliveStatus/activityState/PositionQuality WIP-only, not promoted
- presence_and_age_semantics_v0_1: §4 expanded to 'Not in S03' note (aliveStatus
  unused/stubbed; activityState and PositionQuality policy-only; UI relies on
  is_stale, last_seen_age_s, pos_age_s, posFlags/sats)
- Master table: aliveStatus/activityState/PositionQuality status WIP,
  sent_on_air N, exported_over_ble N, notes 'Not promoted to S03; covered by
  minimal model'
- Regenerate XLSX + CSV

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
+++ b/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>aliveStatus</t>
+          <t>node_id</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -598,23 +598,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>node_id</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>BLE snapshot</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>Y</t>
@@ -622,39 +638,39 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Alive</t>
+          <t>all Node_*</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>alive_packet_encoding_v0 §3.2</t>
+          <t>beacon_payload_encoding_v0 §3</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>OPT</t>
+          <t>MUST</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u48</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>0x00=alive_no_fix</t>
+          <t>6-byte LE MAC48</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>48</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -664,7 +680,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>no-fix liveness</t>
+          <t>every beacon tick</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -676,12 +692,12 @@
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Alive packet optional byte.</t>
+          <t>Primary key; domain uint64 lower 48 bits.</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>Stubbed</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -693,7 +709,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>node_id</t>
+          <t>payloadVersion</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -718,79 +734,71 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>node_id</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>BLE snapshot</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>all Node_*</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>beacon_payload_encoding_v0 §3</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>0x00=v0</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>8</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>all Node_*</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>beacon_payload_encoding_v0 §3</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>u48</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>6-byte LE MAC48</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>48</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -812,7 +820,7 @@
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Primary key; domain uint64 lower 48 bits.</t>
+          <t>Payload format version; first byte of payload.</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -822,14 +830,14 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>payloadVersion</t>
+          <t>positionLat</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -839,7 +847,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -854,23 +862,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>lat_e7</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>BLE snapshot</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
           <t>Y</t>
@@ -878,17 +902,17 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>all Node_*</t>
+          <t>Node_Core_Pos</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>beacon_payload_encoding_v0 §3</t>
+          <t>beacon_payload_encoding_v0 §4.1</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -898,27 +922,19 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u24</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>0x00=v0</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
+          <t>lat_u24 packed; domain 1e-7 deg</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>24</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -928,7 +944,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>every beacon tick</t>
+          <t>every beacon tick when position valid</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -940,7 +956,7 @@
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>Payload format version; first byte of payload.</t>
+          <t>Core only with valid fix. BLE exports lat_e7 (i32).</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -950,14 +966,14 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>positionLat</t>
+          <t>positionLon</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -987,7 +1003,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>lat_e7</t>
+          <t>lon_e7</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1007,7 +1023,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>17</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1047,7 +1063,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>lat_u24 packed; domain 1e-7 deg</t>
+          <t>lon_u24 packed; domain 1e-7 deg</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1076,7 +1092,7 @@
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>Core only with valid fix. BLE exports lat_e7 (i32).</t>
+          <t>Core only with valid fix. BLE exports lon_e7 (i32).</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1093,7 +1109,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>positionLon</t>
+          <t>ref_core_seq16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1103,7 +1119,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1123,7 +1139,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>lon_e7</t>
+          <t>last_core_seq16 (stored); ref in payload</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1133,24 +1149,16 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>stored for Tail-1 match</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1158,17 +1166,17 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Node_Core_Pos</t>
+          <t>Node_Core_Tail</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>beacon_payload_encoding_v0 §4.1</t>
+          <t>tail1_packet_encoding_v0 §3</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1178,29 +1186,29 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>u24</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>lon_u24 packed; domain 1e-7 deg</t>
+          <t>Core linkage key</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>A Core</t>
+          <t>B Tail-1</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>every beacon tick when position valid</t>
+          <t>every Core_Tail</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1212,7 +1220,7 @@
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Core only with valid fix. BLE exports lon_e7 (i32).</t>
+          <t>Back-reference to Core sample seq16; distinct from seq16 in Common.</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1229,7 +1237,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ref_core_seq16</t>
+          <t>seq16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1259,7 +1267,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>last_core_seq16 (stored); ref in payload</t>
+          <t>last_seq</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1269,16 +1277,24 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>stored for Tail-1 match</t>
+          <t>BLE snapshot</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1286,12 +1302,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Node_Core_Tail</t>
+          <t>all Node_*</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>tail1_packet_encoding_v0 §3</t>
+          <t>beacon_payload_encoding_v0 §3; field_cadence_v0 §2</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1311,11 +1327,19 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Core linkage key</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+          <t>LE; global per-node counter</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>65535</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>16</t>
@@ -1323,12 +1347,12 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
+          <t>A Core</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>every Core_Tail</t>
+          <t>every beacon tick</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1340,7 +1364,7 @@
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>Back-reference to Core sample seq16; distinct from seq16 in Common.</t>
+          <t>Dedupe key (nodeId48, seq16). last_seq in NodeEntry.</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1357,17 +1381,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>seq16</t>
+          <t>fwVersionId</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1387,7 +1411,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>last_seq</t>
+          <t>fw_version_id</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1397,47 +1421,39 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>in NodeEntry</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Node_Informative</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>info_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>all Node_*</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>beacon_payload_encoding_v0 §3; field_cadence_v0 §2</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>OPT</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1447,19 +1463,11 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>LE; global per-node counter</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>65535</t>
-        </is>
-      </c>
+          <t>0xFFFF=not present</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>16</t>
@@ -1467,12 +1475,12 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>A Core</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>every beacon tick</t>
+          <t>on change + every 10 min</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -1482,11 +1490,7 @@
       </c>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>Dedupe key (nodeId48, seq16). last_seq in NodeEntry.</t>
-        </is>
-      </c>
+      <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -1494,24 +1498,24 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PositionQuality</t>
+          <t>hwProfileId</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1521,21 +1525,29 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>hw_profile_id</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>in NodeEntry</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>N</t>
@@ -1545,44 +1557,64 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Node_Informative</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>position_quality_v0</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
+          <t>info_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Core + Tail-1 posFlags/sats + age</t>
+          <t>0xFFFF=not present</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>on change + every 10 min</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>Derived; sent components posFlags, sats in Tail-1.</t>
-        </is>
-      </c>
+      <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -1590,19 +1622,19 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>activityState</t>
+          <t>maxSilence10s</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1617,21 +1649,29 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>max_silence_10s</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>in NodeEntry</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
           <t>N</t>
@@ -1641,52 +1681,76 @@
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Node_Informative</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>activity_state_v0</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+          <t>info_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Unknown/Active/Stale/Lost</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
+          <t>10s steps; 0=absent</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>derived on RX</t>
-        </is>
-      </c>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>T_active, T_stale params</t>
-        </is>
-      </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr"/>
+          <t>on change + every 10 min</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>Liveness hint; MUST NOT send on every Operational. Tier C.</t>
+        </is>
+      </c>
       <c r="AC10" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -1694,24 +1758,24 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>fwVersionId</t>
+          <t>lastRxAt</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1721,7 +1785,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1731,7 +1795,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>fw_version_id</t>
+          <t>last_seen_ms</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1741,7 +1805,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>in NodeEntry</t>
+          <t>same as last_seen_ms in code</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1753,64 +1817,52 @@
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Node_Informative</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
-          <t>info_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>link-telemetry-minset-v0 Table A</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>0xFFFF=not present</t>
+          <t>receiver clock</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
+      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>on change + every 10 min</t>
+          <t>on RX</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>periodic</t>
+          <t>event-driven</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>Canon name; firmware uses last_seen_ms.</t>
+        </is>
+      </c>
       <c r="AC11" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -1818,24 +1870,24 @@
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>hwProfileId</t>
+          <t>snrLast</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1845,27 +1897,23 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>hw_profile_id</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>in NodeEntry</t>
+          <t>TODO: add to NodeEntry/BLE if needed</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1877,89 +1925,81 @@
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Node_Informative</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
-          <t>info_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>link_metrics_v0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>0xFFFF=not present</t>
+          <t>dB</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>TODO</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>on change + every 10 min</t>
+          <t>on RX</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>periodic</t>
+          <t>event-driven</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>Not in current BLE record.</t>
+        </is>
+      </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>maxSilence10s</t>
+          <t>batteryPercent</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1979,7 +2019,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>max_silence_10s</t>
+          <t>battery_percent</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2006,12 +2046,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Node_Informative</t>
+          <t>Node_Operational</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>info_packet_encoding_v0 §3.2</t>
+          <t>tail2_packet_encoding_v0 §3.2</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -2031,7 +2071,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>10s steps; 0=absent</t>
+          <t>0-100%; 0xFF=not present</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -2041,12 +2081,12 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>100</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -2056,21 +2096,21 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>on change + every 10 min</t>
+          <t>on change + at forced Core</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>periodic</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr"/>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>battery delta</t>
+        </is>
+      </c>
       <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>Liveness hint; MUST NOT send on every Operational. Tier C.</t>
-        </is>
-      </c>
+      <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -2078,24 +2118,24 @@
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>lastRxAt</t>
+          <t>sats</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2105,7 +2145,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2115,7 +2155,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>last_seen_ms</t>
+          <t>sats</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2125,7 +2165,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>same as last_seen_ms in code</t>
+          <t>in NodeEntry</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -2137,50 +2177,74 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>link-telemetry-minset-v0 Table A</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
+          <t>tail1_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>receiver clock</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
+          <t>satellite count; 0=not present</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>B Tail-1</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>on RX</t>
+          <t>Every Tail-1</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>event-driven</t>
+          <t>periodic</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>Canon name; firmware uses last_seen_ms.</t>
+          <t>v0 canon. In v0.1 packed in pos_quality16; canonical field_key sats.</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
@@ -2190,24 +2254,24 @@
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>snrLast</t>
+          <t>uptimeSec</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2217,23 +2281,27 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>uptime_sec</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>TODO: add to NodeEntry/BLE if needed</t>
+          <t>in NodeEntry</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2245,81 +2313,101 @@
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>link_metrics_v0</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
+          <t>tail2_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>u32</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>dB</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
+          <t>seconds; 0xFFFFFFFF=not present</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>4294967295</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>32</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>B Tail-1</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>on RX</t>
+          <t>on change + at forced Core</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>event-driven</t>
+          <t>periodic+threshold</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>Not in current BLE record.</t>
+          <t>field_cadence: Tier B; packet is Node_Operational (0x04).</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>batteryPercent</t>
+          <t>localAlias</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>LocalOnly</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2329,19 +2417,15 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>AppLocal</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>battery_percent</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2349,7 +2433,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>in NodeEntry</t>
+          <t>app local storage</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2361,76 +2445,40 @@
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Node_Operational</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
-          <t>tail2_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>u8</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>0-100%; 0xFF=not present</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>on change + at forced Core</t>
-        </is>
-      </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>battery delta</t>
-        </is>
-      </c>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>Local phone name; fallback when node_name (authoritative) empty. User-defined on phone; not over radio. Replaced by node-reported node_name when present (authority rule).</t>
+        </is>
+      </c>
       <c r="AC16" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -2438,19 +2486,19 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>pos_age_s</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2460,7 +2508,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>CodeNow</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2475,7 +2523,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>pos_age_s</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2485,49 +2533,45 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>in NodeEntry</t>
+          <t>BLE snapshot</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Node_Core_Tail</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr">
         <is>
-          <t>tail1_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>Tail-1 pos quality; not in Core</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>satellite count; 0=not present</t>
+          <t>seconds</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2537,12 +2581,12 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>65535</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -2550,21 +2594,13 @@
           <t>B Tail-1</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>v0 canon. In v0.1 packed in pos_quality16; canonical field_key sats.</t>
+          <t>S03 minimal. Age of last known position sample (independent from presence). Domain; not in BeaconCore payload (position_quality_v0).</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2581,22 +2617,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>uptimeSec</t>
+          <t>pos_valid</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>CodeNow</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2611,7 +2647,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>uptime_sec</t>
+          <t>pos_valid</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2621,86 +2657,62 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>in NodeEntry</t>
+          <t>BLE snapshot (flags bit1)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Node_Operational</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>tail2_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>u32</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>seconds; 0xFFFFFFFF=not present</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>4294967295</t>
-        </is>
-      </c>
+          <t>flags bit 0x02; Core implies valid</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>on change + at forced Core</t>
-        </is>
-      </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
+          <t>A Core</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>field_cadence: Tier B; packet is Node_Operational (0x04).</t>
+          <t>Domain/BLE only; not on-air in BeaconCore (Core only when fix valid).</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
@@ -2717,27 +2729,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>localAlias</t>
+          <t>is_stale</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LocalOnly</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>CodeNow</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AppLocal</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2748,21 +2760,29 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>app local storage</t>
+          <t>computed at export</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
           <t>N</t>
@@ -2771,20 +2791,28 @@
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>presence_and_age_semantics_v0_1</t>
         </is>
       </c>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr"/>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>flags bit 0x04; last_seen_age_s &gt; expected_interval_s + grace_s</t>
+        </is>
+      </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W19" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -2796,7 +2824,7 @@
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>Local phone name; fallback when node_name (authoritative) empty. User-defined on phone; not over radio. Replaced by node-reported node_name when present (authority rule).</t>
+          <t>S03 minimal. expected_interval_s = max_silence_10s * 10; grace_s hysteresis TBD. Self: TX heartbeat updates last_seen_ms so self does not appear stale (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -2806,24 +2834,24 @@
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>pos_age_s</t>
+          <t>last_seen_age_s</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2833,27 +2861,23 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>pos_age_s</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>computed at export from last_seen_ms</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2863,7 +2887,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2877,11 +2901,7 @@
         </is>
       </c>
       <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Tail-1 pos quality; not in Core</t>
-        </is>
-      </c>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
@@ -2891,27 +2911,15 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>seconds</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>65535</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
+          <t>(now_ms - last_seen_ms)/1000</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X20" t="inlineStr"/>
@@ -2920,7 +2928,7 @@
       <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>S03 minimal. Age of last known position sample (independent from presence). Domain; not in BeaconCore payload (position_quality_v0).</t>
+          <t>S03 minimal. floor((now_ms - last_seen_ms)/1000) at export; BLE convenience; derived from last_seen_ms. See presence_and_age_semantics_v0_1.</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -2930,24 +2938,24 @@
       </c>
       <c r="AD20" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>pos_valid</t>
+          <t>in_use</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>LocalOnly</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2957,7 +2965,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>AppLocal</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2967,34 +2975,26 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>pos_valid</t>
+          <t>in_use</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>BLE snapshot (flags bit1)</t>
+          <t>internal slot only</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>N</t>
@@ -3009,21 +3009,13 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>flags bit 0x02; Core implies valid</t>
-        </is>
-      </c>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr">
         <is>
-          <t>A Core</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X21" t="inlineStr"/>
@@ -3032,7 +3024,7 @@
       <c r="AA21" t="inlineStr"/>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>Domain/BLE only; not on-air in BeaconCore (Core only when fix valid).</t>
+          <t>Internal; not in BLE.</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
@@ -3042,24 +3034,24 @@
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>is_stale</t>
+          <t>is_self</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>LocalOnly</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3069,23 +3061,27 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>AppLocal</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>is_self</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>computed at export</t>
+          <t>BLE snapshot (flags bit0)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -3109,11 +3105,7 @@
         </is>
       </c>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>presence_and_age_semantics_v0_1</t>
-        </is>
-      </c>
+      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
@@ -3123,7 +3115,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>flags bit 0x04; last_seen_age_s &gt; expected_interval_s + grace_s</t>
+          <t>flags bit 0x01</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3142,11 +3134,7 @@
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr">
-        <is>
-          <t>S03 minimal. expected_interval_s = max_silence_10s * 10; grace_s hysteresis TBD. Self: TX heartbeat updates last_seen_ms so self does not appear stale (presence_and_age_semantics_v0_1).</t>
-        </is>
-      </c>
+      <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3154,19 +3142,19 @@
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>last_seen_age_s</t>
+          <t>last_applied_tail_ref_core_seq16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3181,47 +3169,43 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>last_applied_tail_ref_core_seq16</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>computed at export from last_seen_ms</t>
-        </is>
-      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>tail1_packet_encoding_v0; at most one Tail per Core</t>
+        </is>
+      </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
@@ -3229,11 +3213,7 @@
           <t>u16</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>(now_ms - last_seen_ms)/1000</t>
-        </is>
-      </c>
+      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
@@ -3248,7 +3228,7 @@
       <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>S03 minimal. floor((now_ms - last_seen_ms)/1000) at export; BLE convenience; derived from last_seen_ms. See presence_and_age_semantics_v0_1.</t>
+          <t>Variant 2: dedupe second Tail-1 for same ref_core_seq16.</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -3265,7 +3245,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>in_use</t>
+          <t>short_id</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3275,7 +3255,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LocalOnly</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3285,7 +3265,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AppLocal</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3295,26 +3275,34 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>in_use</t>
+          <t>short_id</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>internal slot only</t>
+          <t>BLE snapshot</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M24" t="inlineStr">
         <is>
           <t>N</t>
@@ -3326,13 +3314,21 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr"/>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>CRC16-CCITT over node_id LE</t>
+        </is>
+      </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="W24" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3344,7 +3340,7 @@
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>Internal; not in BLE.</t>
+          <t>Display only; not protocol key. Reserved 0x0000/0xFFFF handled.</t>
         </is>
       </c>
       <c r="AC24" t="inlineStr">
@@ -3361,7 +3357,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>is_self</t>
+          <t>short_id_collision</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3371,7 +3367,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LocalOnly</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3381,7 +3377,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AppLocal</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3391,7 +3387,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>is_self</t>
+          <t>short_id_collision</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3401,7 +3397,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BLE snapshot (flags bit0)</t>
+          <t>BLE snapshot (flags bit3)</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -3435,7 +3431,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>flags bit 0x01</t>
+          <t>flags bit 0x08</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -3462,24 +3458,24 @@
       </c>
       <c r="AD25" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>last_applied_tail_ref_core_seq16</t>
+          <t>last_rx_rssi</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3499,22 +3495,34 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>last_applied_tail_ref_core_seq16</t>
+          <t>last_rx_rssi</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>BLE snapshot</t>
+        </is>
+      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M26" t="inlineStr">
         <is>
           <t>N</t>
@@ -3523,32 +3531,48 @@
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
-          <t>tail1_packet_encoding_v0; at most one Tail per Core</t>
+          <t>link_metrics_v0</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>u16</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr"/>
+          <t>i8</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>dBm</t>
+        </is>
+      </c>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W26" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>on RX</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>event-driven</t>
+        </is>
+      </c>
       <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="inlineStr"/>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>Variant 2: dedupe second Tail-1 for same ref_core_seq16.</t>
+          <t>rssiLast; receiver-side only.</t>
         </is>
       </c>
       <c r="AC26" t="inlineStr">
@@ -3558,24 +3582,24 @@
       </c>
       <c r="AD26" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>short_id</t>
+          <t>last_seen_ms</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3585,7 +3609,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3595,7 +3619,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>short_id</t>
+          <t>last_seen_ms</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3605,24 +3629,16 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>internal; BLE exports last_seen_age_s derived</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
           <t>N</t>
@@ -3634,33 +3650,37 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>u32</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>CRC16-CCITT over node_id LE</t>
+          <t>uptime ms</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
+      <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>on RX</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>event-driven</t>
+        </is>
+      </c>
       <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="inlineStr"/>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>Display only; not protocol key. Reserved 0x0000/0xFFFF handled.</t>
+          <t>Exported as lastSeenAgeS (age_s) in BLE.</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr">
@@ -3670,19 +3690,19 @@
       </c>
       <c r="AD27" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>short_id_collision</t>
+          <t>networkName</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3692,115 +3712,95 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>CodeNow</t>
+          <t>Idea</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>short_id_collision</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>BLE snapshot (flags bit3)</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>index §4</t>
+        </is>
+      </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>flags bit 0x08</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr">
-        <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr"/>
-      <c r="AB28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>Out-of-scope S03; NOT sent in v0 beacon; future session-join.</t>
+        </is>
+      </c>
       <c r="AC28" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD28" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>last_rx_rssi</t>
+          <t>hops</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Routing/Mesh</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CodeNow</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -3810,39 +3810,23 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>last_rx_rssi</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>BLE snapshot</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>N</t>
@@ -3851,80 +3835,68 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
-          <t>link_metrics_v0</t>
+          <t>meshtastic-nodetable.md §3</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>i8</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>dBm</t>
+          <t>hops_away</t>
         </is>
       </c>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+      <c r="V29" t="inlineStr"/>
       <c r="W29" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
-        <is>
-          <t>on RX</t>
-        </is>
-      </c>
-      <c r="Y29" t="inlineStr">
-        <is>
-          <t>event-driven</t>
-        </is>
-      </c>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
       <c r="AA29" t="inlineStr"/>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>rssiLast; receiver-side only.</t>
+          <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD29" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>last_seen_ms</t>
+          <t>last_direct_time</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CodeNow</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -3934,24 +3906,16 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>last_seen_ms</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>internal; BLE exports last_seen_age_s derived</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>N</t>
@@ -3965,19 +3929,19 @@
         </is>
       </c>
       <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>naviga_mesh_protocol_concept_v1_4.md</t>
+        </is>
+      </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>u32</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>uptime ms</t>
-        </is>
-      </c>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr"/>
@@ -3986,26 +3950,18 @@
           <t>Derived/Injected</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>on RX</t>
-        </is>
-      </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>event-driven</t>
-        </is>
-      </c>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>Exported as lastSeenAgeS (age_s) in BLE.</t>
+          <t>Time of last direct RX from this node; mesh concept. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD30" t="inlineStr">
@@ -4017,27 +3973,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>networkName</t>
+          <t>next_hop</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Routing/Mesh</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4067,28 +4023,36 @@
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr">
         <is>
-          <t>index §4</t>
+          <t>meshtastic-nodetable.md §3</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>last byte of node num</t>
+        </is>
+      </c>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
       <c r="X31" t="inlineStr"/>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>Out-of-scope S03; NOT sent in v0 beacon; future session-join.</t>
+          <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -4098,14 +4062,14 @@
       </c>
       <c r="AD31" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>hops</t>
+          <t>pos_history</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4115,7 +4079,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Routing/Mesh</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4125,7 +4089,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4155,19 +4119,19 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
-          <t>meshtastic-nodetable.md §3</t>
+          <t>naviga_mesh_protocol_concept_v1_4.md</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>array</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>hops_away</t>
+          <t>short history of positions</t>
         </is>
       </c>
       <c r="T32" t="inlineStr"/>
@@ -4184,7 +4148,7 @@
       <c r="AA32" t="inlineStr"/>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>No mesh routing in Naviga v0.</t>
+          <t>Optional pos_history_X; mesh concept. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -4194,14 +4158,14 @@
       </c>
       <c r="AD32" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>last_direct_time</t>
+          <t>role_params</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4211,7 +4175,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4221,7 +4185,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4258,10 +4222,14 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr"/>
+          <t>enum/params</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>role_pos_update_interval_X etc</t>
+        </is>
+      </c>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
@@ -4276,7 +4244,7 @@
       <c r="AA33" t="inlineStr"/>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>Time of last direct RX from this node; mesh concept. Non-goal v0.</t>
+          <t>Role-based delivery params; mesh concept. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC33" t="inlineStr">
@@ -4286,14 +4254,14 @@
       </c>
       <c r="AD33" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>next_hop</t>
+          <t>rssi_direct</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4303,7 +4271,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Routing/Mesh</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4343,21 +4311,17 @@
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr">
         <is>
-          <t>meshtastic-nodetable.md §3</t>
+          <t>meshtastic research</t>
         </is>
       </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>u8</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>last byte of node num</t>
-        </is>
-      </c>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="inlineStr"/>
@@ -4372,7 +4336,7 @@
       <c r="AA34" t="inlineStr"/>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>No mesh routing in Naviga v0.</t>
+          <t>Direct-link RSSI; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC34" t="inlineStr">
@@ -4382,14 +4346,14 @@
       </c>
       <c r="AD34" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>pos_history</t>
+          <t>snr_direct</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4399,7 +4363,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4409,7 +4373,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4439,21 +4403,17 @@
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr">
         <is>
-          <t>naviga_mesh_protocol_concept_v1_4.md</t>
+          <t>meshtastic research</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>short history of positions</t>
-        </is>
-      </c>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="inlineStr"/>
@@ -4468,7 +4428,7 @@
       <c r="AA35" t="inlineStr"/>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>Optional pos_history_X; mesh concept. Non-goal v0.</t>
+          <t>Direct-link SNR; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC35" t="inlineStr">
@@ -4478,19 +4438,19 @@
       </c>
       <c r="AD35" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>role_params</t>
+          <t>is_grey</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4500,12 +4460,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4522,37 +4482,45 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>naviga_mesh_protocol_concept_v1_4.md</t>
-        </is>
-      </c>
+      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>enum/params</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>role_pos_update_interval_X etc</t>
+          <t>same as is_stale (flags bit 0x04)</t>
         </is>
       </c>
       <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr"/>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W36" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -4564,58 +4532,66 @@
       <c r="AA36" t="inlineStr"/>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>Role-based delivery params; mesh concept. Non-goal v0.</t>
+          <t>Alias; superseded-by is_stale (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC36" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD36" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>rssi_direct</t>
+          <t>posFlags</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>pos_flags</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>in NodeEntry</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr">
         <is>
           <t>N</t>
@@ -4625,75 +4601,111 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>meshtastic research</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
+          <t>tail1_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>bit0=position valid; 1-7 reserved</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="inlineStr"/>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z37" t="inlineStr"/>
       <c r="AA37" t="inlineStr"/>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>Direct-link RSSI; Mesh_future. Non-goal v0.</t>
+          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD37" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>snr_direct</t>
+          <t>pos_sats</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4723,23 +4735,27 @@
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr">
         <is>
-          <t>meshtastic research</t>
+          <t>packet_sets_v0_1</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>alias for sats</t>
+        </is>
+      </c>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>B Tail-1</t>
         </is>
       </c>
       <c r="X38" t="inlineStr"/>
@@ -4748,7 +4764,7 @@
       <c r="AA38" t="inlineStr"/>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>Direct-link SNR; Mesh_future. Non-goal v0.</t>
+          <t>Alias; superseded-by sats.</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
@@ -4758,19 +4774,19 @@
       </c>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>is_grey</t>
+          <t>aliveStatus</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4780,12 +4796,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Superseded</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4802,79 +4818,95 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Alive</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>alive_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>same as is_stale (flags bit 0x04)</t>
+          <t>0x00=alive_no_fix</t>
         </is>
       </c>
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr"/>
-      <c r="Y39" t="inlineStr"/>
+          <t>A Core</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>no-fix liveness</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>Alias; superseded-by is_stale (presence_and_age_semantics_v0_1).</t>
+          <t>Not promoted to S03; unused/stubbed. Covered by minimal model (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Stubbed</t>
         </is>
       </c>
       <c r="AD39" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>posFlags</t>
+          <t>PositionQuality</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4884,34 +4916,26 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Superseded</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>pos_flags</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>in NodeEntry</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>N</t>
@@ -4921,111 +4945,79 @@
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>Node_Core_Tail</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
-          <t>tail1_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>position_quality_v0</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>bit0=position valid; 1-7 reserved</t>
-        </is>
-      </c>
-      <c r="T40" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="V40" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+          <t>Core + Tail-1 posFlags/sats + age</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr"/>
       <c r="W40" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X40" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y40" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr"/>
+      <c r="Y40" t="inlineStr"/>
       <c r="Z40" t="inlineStr"/>
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
+          <t>Not promoted to S03; policy-only derived. Covered by minimal model (pos_age_s, posFlags/sats; presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC40" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD40" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>pos_sats</t>
+          <t>activityState</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Superseded</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -5055,19 +5047,19 @@
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
-          <t>packet_sets_v0_1</t>
+          <t>activity_state_v0</t>
         </is>
       </c>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>alias for sats</t>
+          <t>Unknown/Active/Stale/Lost</t>
         </is>
       </c>
       <c r="T41" t="inlineStr"/>
@@ -5075,16 +5067,24 @@
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X41" t="inlineStr"/>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>derived on RX</t>
+        </is>
+      </c>
       <c r="Y41" t="inlineStr"/>
-      <c r="Z41" t="inlineStr"/>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>T_active, T_stale params</t>
+        </is>
+      </c>
       <c r="AA41" t="inlineStr"/>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>Alias; superseded-by sats.</t>
+          <t>Not promoted to S03; policy-only derived. Covered by minimal model (is_stale, last_seen_age_s; presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC41" t="inlineStr">

</xml_diff>

<commit_message>
S03 WIP: seq/ref/version/link-metrics block
- Add seq_ref_version_link_metrics_v0_1.md: definitions (last_seq16,
  last_core_seq16, ref_core_seq16, last_applied_tail_ref_core_seq16),
  link metrics (last_rx_rssi, snrLast E22 NA sentinel), payloadVersion
  -> last_payload_version_seen (injected, debug only), update rules
- Master table: last_payload_version_seen (WIP, Injected); payloadVersion
  note; seq16/ref_core_seq16/last_applied_tail/last_rx_rssi/snrLast notes
  and seq_ref_version_link_metrics_v0_1 refs
- Regenerate XLSX + CSV; add SOURCES entry

Refs #351 #352. Follow-up: #375 (RSSI), #376 (snrLast sentinel).

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
+++ b/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD55"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -820,7 +820,7 @@
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Payload format version; first byte of payload.</t>
+          <t>On-air: first byte of payload. NodeTable/store may use last_payload_version_seen (injected, debug only). seq_ref_version_link_metrics_v0_1.</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -1220,7 +1220,7 @@
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Back-reference to Core sample seq16; distinct from seq16 in Common.</t>
+          <t>Tail-only ref. Back-reference to Core sample seq16. last_core_seq16 updates only on Core_Pos RX; tail apply only on Tail RX (seq_ref_version_link_metrics_v0_1).</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1364,7 +1364,7 @@
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>Dedupe key (nodeId48, seq16). last_seq in NodeEntry.</t>
+          <t>Dedupe key (nodeId48, seq16). last_seq in NodeEntry. Updates on any RX. last_core_seq16 updates only on Core_Pos RX; tail ref/apply only on Tail RX (seq_ref_version_link_metrics_v0_1).</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1877,17 +1877,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>snrLast</t>
+          <t>batteryPercent</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1897,23 +1897,27 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>battery_percent</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>TODO: add to NodeEntry/BLE if needed</t>
+          <t>in NodeEntry</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1925,71 +1929,91 @@
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>link_metrics_v0</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+          <t>tail2_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>dB</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
+          <t>0-100%; 0xFF=not present</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>7</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>on RX</t>
+          <t>on change + at forced Core</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>event-driven</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr"/>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>battery delta</t>
+        </is>
+      </c>
       <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>Not in current BLE record.</t>
-        </is>
-      </c>
+      <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>batteryPercent</t>
+          <t>sats</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1999,7 +2023,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2019,7 +2043,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>battery_percent</t>
+          <t>sats</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2046,12 +2070,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Node_Operational</t>
+          <t>Node_Core_Tail</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>tail2_packet_encoding_v0 §3.2</t>
+          <t>tail1_packet_encoding_v0 §3.2</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -2071,7 +2095,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>0-100%; 0xFF=not present</t>
+          <t>satellite count; 0=not present</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -2081,36 +2105,36 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>255</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
+          <t>B Tail-1</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>on change + at forced Core</t>
+          <t>Every Tail-1</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>battery delta</t>
-        </is>
-      </c>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>v0 canon. In v0.1 packed in pos_quality16; canonical field_key sats.</t>
+        </is>
+      </c>
       <c r="AC13" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -2125,7 +2149,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>uptimeSec</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2135,7 +2159,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2155,7 +2179,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>uptime_sec</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2182,17 +2206,17 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Node_Core_Tail</t>
+          <t>Node_Operational</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>tail1_packet_encoding_v0 §3.2</t>
+          <t>tail2_packet_encoding_v0 §3.2</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -2202,12 +2226,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u32</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>satellite count; 0=not present</t>
+          <t>seconds; 0xFFFFFFFF=not present</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -2217,12 +2241,12 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>4294967295</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>32</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -2232,19 +2256,19 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>Every Tail-1</t>
+          <t>on change + at forced Core</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>periodic</t>
+          <t>periodic+threshold</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>v0 canon. In v0.1 packed in pos_quality16; canonical field_key sats.</t>
+          <t>field_cadence: Tier B; packet is Node_Operational (0x04).</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
@@ -2261,17 +2285,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>uptimeSec</t>
+          <t>localAlias</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>LocalOnly</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2281,19 +2305,15 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>AppLocal</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>uptime_sec</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2301,7 +2321,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>in NodeEntry</t>
+          <t>app local storage</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2313,74 +2333,38 @@
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Node_Operational</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
-          <t>tail2_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>u32</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>seconds; 0xFFFFFFFF=not present</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>4294967295</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>on change + at forced Core</t>
-        </is>
-      </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>field_cadence: Tier B; packet is Node_Operational (0x04).</t>
+          <t>Local phone name; fallback when node_name (authoritative) empty. User-defined on phone; not over radio. Replaced by node-reported node_name when present (authority rule).</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -2390,42 +2374,46 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>localAlias</t>
+          <t>pos_age_s</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LocalOnly</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>CodeNow</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>AppLocal</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>pos_age_s</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2433,16 +2421,24 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>app local storage</t>
+          <t>BLE snapshot</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
           <t>N</t>
@@ -2451,23 +2447,39 @@
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>Tail-1 pos quality; not in Core</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>65535</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>B Tail-1</t>
         </is>
       </c>
       <c r="X16" t="inlineStr"/>
@@ -2476,7 +2488,7 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>Local phone name; fallback when node_name (authoritative) empty. User-defined on phone; not over radio. Replaced by node-reported node_name when present (authority rule).</t>
+          <t>S03 minimal. Age of last known position sample (independent from presence). Domain; not in BeaconCore payload (position_quality_v0).</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
@@ -2486,14 +2498,14 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>pos_age_s</t>
+          <t>pos_valid</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2523,7 +2535,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>pos_age_s</t>
+          <t>pos_valid</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2533,7 +2545,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>BLE snapshot (flags bit1)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2543,12 +2555,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2557,41 +2569,29 @@
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Tail-1 pos quality; not in Core</t>
-        </is>
-      </c>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>seconds</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>65535</t>
-        </is>
-      </c>
+          <t>flags bit 0x02; Core implies valid</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
+          <t>A Core</t>
         </is>
       </c>
       <c r="X17" t="inlineStr"/>
@@ -2600,7 +2600,7 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>S03 minimal. Age of last known position sample (independent from presence). Domain; not in BeaconCore payload (position_quality_v0).</t>
+          <t>Domain/BLE only; not on-air in BeaconCore (Core only when fix valid).</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2617,17 +2617,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>pos_valid</t>
+          <t>is_stale</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2637,27 +2637,23 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>pos_valid</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>BLE snapshot (flags bit1)</t>
+          <t>computed at export</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2681,7 +2677,11 @@
         </is>
       </c>
       <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>presence_and_age_semantics_v0_1</t>
+        </is>
+      </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>flags bit 0x02; Core implies valid</t>
+          <t>flags bit 0x04; last_seen_age_s &gt; expected_interval_s + grace_s</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -2703,7 +2703,7 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>A Core</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X18" t="inlineStr"/>
@@ -2712,7 +2712,7 @@
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>Domain/BLE only; not on-air in BeaconCore (Core only when fix valid).</t>
+          <t>S03 minimal. expected_interval_s = max_silence_10s * 10; grace_s hysteresis TBD. Self: TX heartbeat updates last_seen_ms so self does not appear stale (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
@@ -2722,14 +2722,14 @@
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>is_stale</t>
+          <t>last_seen_age_s</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>computed at export</t>
+          <t>computed at export from last_seen_ms</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2775,12 +2775,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2789,30 +2789,22 @@
         </is>
       </c>
       <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>presence_and_age_semantics_v0_1</t>
-        </is>
-      </c>
+      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>flags bit 0x04; last_seen_age_s &gt; expected_interval_s + grace_s</t>
+          <t>(now_ms - last_seen_ms)/1000</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -2824,7 +2816,7 @@
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>S03 minimal. expected_interval_s = max_silence_10s * 10; grace_s hysteresis TBD. Self: TX heartbeat updates last_seen_ms so self does not appear stale (presence_and_age_semantics_v0_1).</t>
+          <t>S03 minimal. floor((now_ms - last_seen_ms)/1000) at export; BLE convenience; derived from last_seen_ms. See presence_and_age_semantics_v0_1.</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -2841,17 +2833,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>last_seen_age_s</t>
+          <t>in_use</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>LocalOnly</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2861,15 +2853,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>AppLocal</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>in_use</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>N</t>
@@ -2877,24 +2873,16 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>computed at export from last_seen_ms</t>
+          <t>internal slot only</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>N</t>
@@ -2906,14 +2894,10 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>u16</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>(now_ms - last_seen_ms)/1000</t>
-        </is>
-      </c>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
@@ -2928,7 +2912,7 @@
       <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>S03 minimal. floor((now_ms - last_seen_ms)/1000) at export; BLE convenience; derived from last_seen_ms. See presence_and_age_semantics_v0_1.</t>
+          <t>Internal; not in BLE.</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -2945,7 +2929,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>in_use</t>
+          <t>is_self</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2975,26 +2959,34 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>in_use</t>
+          <t>is_self</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>internal slot only</t>
+          <t>BLE snapshot (flags bit0)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>N</t>
@@ -3009,10 +3001,18 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>flags bit 0x01</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W21" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3022,11 +3022,7 @@
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr"/>
-      <c r="AB21" t="inlineStr">
-        <is>
-          <t>Internal; not in BLE.</t>
-        </is>
-      </c>
+      <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3034,14 +3030,14 @@
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>is_self</t>
+          <t>last_applied_tail_ref_core_seq16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3051,7 +3047,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LocalOnly</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3061,7 +3057,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AppLocal</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3071,60 +3067,44 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>is_self</t>
+          <t>last_applied_tail_ref_core_seq16</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>BLE snapshot (flags bit0)</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>tail1_packet_encoding_v0; at most one Tail per Core</t>
+        </is>
+      </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>flags bit 0x01</t>
-        </is>
-      </c>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3134,7 +3114,11 @@
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>Variant 2: dedupe second Tail-1 for same ref_core_seq16. Updates only on Tail RX when applied (seq_ref_version_link_metrics_v0_1).</t>
+        </is>
+      </c>
       <c r="AC22" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3142,14 +3126,14 @@
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>last_applied_tail_ref_core_seq16</t>
+          <t>short_id</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3159,7 +3143,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3169,7 +3153,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3179,33 +3163,41 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>last_applied_tail_ref_core_seq16</t>
+          <t>short_id</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>BLE snapshot</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>tail1_packet_encoding_v0; at most one Tail per Core</t>
-        </is>
-      </c>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
@@ -3213,10 +3205,18 @@
           <t>u16</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>CRC16-CCITT over node_id LE</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="W23" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3228,7 +3228,7 @@
       <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>Variant 2: dedupe second Tail-1 for same ref_core_seq16.</t>
+          <t>Display only; not protocol key. Reserved 0x0000/0xFFFF handled.</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -3245,7 +3245,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>short_id</t>
+          <t>short_id_collision</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>short_id</t>
+          <t>short_id_collision</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>BLE snapshot (flags bit3)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -3295,12 +3295,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3314,19 +3314,19 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>CRC16-CCITT over node_id LE</t>
+          <t>flags bit 0x08</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
@@ -3338,11 +3338,7 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr">
-        <is>
-          <t>Display only; not protocol key. Reserved 0x0000/0xFFFF handled.</t>
-        </is>
-      </c>
+      <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3357,17 +3353,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>short_id_collision</t>
+          <t>last_rx_rssi</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3377,7 +3373,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3387,7 +3383,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>short_id_collision</t>
+          <t>last_rx_rssi</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3397,7 +3393,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BLE snapshot (flags bit3)</t>
+          <t>BLE snapshot</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -3407,7 +3403,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>23</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -3421,24 +3417,28 @@
         </is>
       </c>
       <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>link_metrics_v0</t>
+        </is>
+      </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>i8</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>flags bit 0x08</t>
+          <t>dBm</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
@@ -3446,11 +3446,23 @@
           <t>Derived/Injected</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>on RX</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>event-driven</t>
+        </is>
+      </c>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>S03 required. rssiLast; updated on any RX from that node. Units raw or dBm TBD. seq_ref_version_link_metrics_v0_1.</t>
+        </is>
+      </c>
       <c r="AC25" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3458,14 +3470,14 @@
       </c>
       <c r="AD25" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>last_rx_rssi</t>
+          <t>last_seen_ms</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3475,7 +3487,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3495,7 +3507,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>last_rx_rssi</t>
+          <t>last_seen_ms</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3505,54 +3517,38 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>internal; BLE exports last_seen_age_s derived</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>link_metrics_v0</t>
-        </is>
-      </c>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>i8</t>
+          <t>u32</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>dBm</t>
+          <t>uptime ms</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3572,7 +3568,7 @@
       <c r="AA26" t="inlineStr"/>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>rssiLast; receiver-side only.</t>
+          <t>Exported as lastSeenAgeS (age_s) in BLE.</t>
         </is>
       </c>
       <c r="AC26" t="inlineStr">
@@ -3589,49 +3585,41 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>last_seen_ms</t>
+          <t>networkName</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CodeNow</t>
+          <t>Idea</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>last_seen_ms</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>internal; BLE exports last_seen_age_s derived</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>N</t>
@@ -3645,79 +3633,67 @@
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>index §4</t>
+        </is>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>u32</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>uptime ms</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>on RX</t>
-        </is>
-      </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>event-driven</t>
-        </is>
-      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="inlineStr"/>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>Exported as lastSeenAgeS (age_s) in BLE.</t>
+          <t>Out-of-scope S03; NOT sent in v0 beacon; future session-join.</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>networkName</t>
+          <t>hops</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Routing/Mesh</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3747,28 +3723,36 @@
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
-          <t>index §4</t>
+          <t>meshtastic-nodetable.md §3</t>
         </is>
       </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>hops_away</t>
+        </is>
+      </c>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr"/>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>Out-of-scope S03; NOT sent in v0 beacon; future session-join.</t>
+          <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
       <c r="AC28" t="inlineStr">
@@ -3778,14 +3762,14 @@
       </c>
       <c r="AD28" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>hops</t>
+          <t>last_direct_time</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3795,7 +3779,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Routing/Mesh</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3835,21 +3819,17 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
-          <t>meshtastic-nodetable.md §3</t>
+          <t>naviga_mesh_protocol_concept_v1_4.md</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>u8</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>hops_away</t>
-        </is>
-      </c>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
@@ -3864,7 +3844,7 @@
       <c r="AA29" t="inlineStr"/>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>No mesh routing in Naviga v0.</t>
+          <t>Time of last direct RX from this node; mesh concept. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC29" t="inlineStr">
@@ -3874,14 +3854,14 @@
       </c>
       <c r="AD29" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>last_direct_time</t>
+          <t>next_hop</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3891,7 +3871,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Routing/Mesh</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3931,17 +3911,21 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr">
         <is>
-          <t>naviga_mesh_protocol_concept_v1_4.md</t>
+          <t>meshtastic-nodetable.md §3</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>last byte of node num</t>
+        </is>
+      </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr"/>
@@ -3956,7 +3940,7 @@
       <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>Time of last direct RX from this node; mesh concept. Non-goal v0.</t>
+          <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
@@ -3966,14 +3950,14 @@
       </c>
       <c r="AD30" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>next_hop</t>
+          <t>pos_history</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3983,7 +3967,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Routing/Mesh</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3993,7 +3977,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4023,19 +4007,19 @@
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr">
         <is>
-          <t>meshtastic-nodetable.md §3</t>
+          <t>naviga_mesh_protocol_concept_v1_4.md</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>array</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>last byte of node num</t>
+          <t>short history of positions</t>
         </is>
       </c>
       <c r="T31" t="inlineStr"/>
@@ -4052,7 +4036,7 @@
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>No mesh routing in Naviga v0.</t>
+          <t>Optional pos_history_X; mesh concept. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -4062,14 +4046,14 @@
       </c>
       <c r="AD31" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>pos_history</t>
+          <t>role_params</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4079,7 +4063,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4126,12 +4110,12 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>enum/params</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>short history of positions</t>
+          <t>role_pos_update_interval_X etc</t>
         </is>
       </c>
       <c r="T32" t="inlineStr"/>
@@ -4148,7 +4132,7 @@
       <c r="AA32" t="inlineStr"/>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>Optional pos_history_X; mesh concept. Non-goal v0.</t>
+          <t>Role-based delivery params; mesh concept. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -4158,14 +4142,14 @@
       </c>
       <c r="AD32" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>role_params</t>
+          <t>rssi_direct</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4175,7 +4159,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4185,7 +4169,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4215,21 +4199,17 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>naviga_mesh_protocol_concept_v1_4.md</t>
+          <t>meshtastic research</t>
         </is>
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>enum/params</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>role_pos_update_interval_X etc</t>
-        </is>
-      </c>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
@@ -4244,7 +4224,7 @@
       <c r="AA33" t="inlineStr"/>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>Role-based delivery params; mesh concept. Non-goal v0.</t>
+          <t>Direct-link RSSI; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC33" t="inlineStr">
@@ -4254,14 +4234,14 @@
       </c>
       <c r="AD33" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>rssi_direct</t>
+          <t>snr_direct</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4336,7 +4316,7 @@
       <c r="AA34" t="inlineStr"/>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>Direct-link RSSI; Mesh_future. Non-goal v0.</t>
+          <t>Direct-link SNR; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC34" t="inlineStr">
@@ -4353,27 +4333,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>snr_direct</t>
+          <t>is_grey</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4390,33 +4370,45 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>meshtastic research</t>
-        </is>
-      </c>
+      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr"/>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>same as is_stale (flags bit 0x04)</t>
+        </is>
+      </c>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W35" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -4428,34 +4420,34 @@
       <c r="AA35" t="inlineStr"/>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>Direct-link SNR; Mesh_future. Non-goal v0.</t>
+          <t>Alias; superseded-by is_stale (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC35" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD35" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>is_grey</t>
+          <t>posFlags</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4465,74 +4457,106 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>pos_flags</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>in NodeEntry</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>tail1_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>same as is_stale (flags bit 0x04)</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
+          <t>bit0=position valid; 1-7 reserved</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X36" t="inlineStr"/>
-      <c r="Y36" t="inlineStr"/>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z36" t="inlineStr"/>
       <c r="AA36" t="inlineStr"/>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>Alias; superseded-by is_stale (presence_and_age_semantics_v0_1).</t>
+          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
         </is>
       </c>
       <c r="AC36" t="inlineStr">
@@ -4542,14 +4566,14 @@
       </c>
       <c r="AD36" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>posFlags</t>
+          <t>pos_sats</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4574,24 +4598,16 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>pos_flags</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>in NodeEntry</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>N</t>
@@ -4601,29 +4617,17 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Node_Core_Tail</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr">
         <is>
-          <t>tail1_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
           <t>u8</t>
@@ -4631,76 +4635,56 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>bit0=position valid; 1-7 reserved</t>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+          <t>alias for sats</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr">
         <is>
           <t>B Tail-1</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y37" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="inlineStr"/>
       <c r="AA37" t="inlineStr"/>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
+          <t>Alias; superseded-by sats.</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD37" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>pos_sats</t>
+          <t>aliveStatus</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Superseded</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4732,14 +4716,26 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Alive</t>
+        </is>
+      </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>packet_sets_v0_1</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
+          <t>alive_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R38" t="inlineStr">
         <is>
           <t>u8</t>
@@ -4747,51 +4743,63 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>alias for sats</t>
+          <t>0x00=alive_no_fix</t>
         </is>
       </c>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X38" t="inlineStr"/>
-      <c r="Y38" t="inlineStr"/>
+          <t>A Core</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>no-fix liveness</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z38" t="inlineStr"/>
       <c r="AA38" t="inlineStr"/>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>Alias; superseded-by sats.</t>
+          <t>Not promoted to S03; unused/stubbed. Covered by minimal model (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Stubbed</t>
         </is>
       </c>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>aliveStatus</t>
+          <t>PositionQuality</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4801,7 +4809,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4828,80 +4836,56 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Alive</t>
-        </is>
-      </c>
+      <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr">
         <is>
-          <t>alive_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>position_quality_v0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>0x00=alive_no_fix</t>
+          <t>Core + Tail-1 posFlags/sats + age</t>
         </is>
       </c>
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+      <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr">
         <is>
-          <t>A Core</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>no-fix liveness</t>
-        </is>
-      </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>Not promoted to S03; unused/stubbed. Covered by minimal model (presence_and_age_semantics_v0_1).</t>
+          <t>Not promoted to S03; policy-only derived. Covered by minimal model (pos_age_s, posFlags/sats; presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>Stubbed</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD39" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PositionQuality</t>
+          <t>activityState</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4911,7 +4895,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4951,19 +4935,19 @@
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
-          <t>position_quality_v0</t>
+          <t>activity_state_v0</t>
         </is>
       </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Core + Tail-1 posFlags/sats + age</t>
+          <t>Unknown/Active/Stale/Lost</t>
         </is>
       </c>
       <c r="T40" t="inlineStr"/>
@@ -4974,13 +4958,21 @@
           <t>Derived/Injected</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr"/>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>derived on RX</t>
+        </is>
+      </c>
       <c r="Y40" t="inlineStr"/>
-      <c r="Z40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>T_active, T_stale params</t>
+        </is>
+      </c>
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>Not promoted to S03; policy-only derived. Covered by minimal model (pos_age_s, posFlags/sats; presence_and_age_semantics_v0_1).</t>
+          <t>Not promoted to S03; policy-only derived. Covered by minimal model (is_stale, last_seen_age_s; presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC40" t="inlineStr">
@@ -4997,17 +4989,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>activityState</t>
+          <t>role_id</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5017,7 +5009,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -5041,50 +5033,62 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Node_Informative</t>
+        </is>
+      </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>activity_state_v0</t>
+          <t>packet_sets_v0_1</t>
         </is>
       </c>
       <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Unknown/Active/Stale/Lost</t>
+          <t>role identifier</t>
         </is>
       </c>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>derived on RX</t>
-        </is>
-      </c>
-      <c r="Y41" t="inlineStr"/>
-      <c r="Z41" t="inlineStr">
-        <is>
-          <t>T_active, T_stale params</t>
-        </is>
-      </c>
+          <t>periodic + changed-boost</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr"/>
       <c r="AA41" t="inlineStr"/>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>Not promoted to S03; policy-only derived. Covered by minimal model (is_stale, last_seen_age_s; presence_and_age_semantics_v0_1).</t>
+          <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
         </is>
       </c>
       <c r="AC41" t="inlineStr">
@@ -5094,19 +5098,19 @@
       </c>
       <c r="AD41" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>role_id</t>
+          <t>last_payload_version_seen</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5121,7 +5125,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5135,7 +5139,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>debug only; not persisted</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr">
         <is>
           <t>N</t>
@@ -5145,25 +5153,17 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Node_Informative</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr">
         <is>
-          <t>packet_sets_v0_1</t>
+          <t>seq_ref_version_link_metrics_v0_1</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>u8</t>
@@ -5171,36 +5171,36 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>role identifier</t>
+          <t>last seen payloadVersion byte</t>
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>periodic + changed-boost</t>
+          <t>on RX</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>periodic</t>
+          <t>event-driven</t>
         </is>
       </c>
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
+          <t>Injected; decoder/debug aid only. Not user-facing; not persisted. Optional in NodeEntry. seq_ref_version_link_metrics_v0_1.</t>
         </is>
       </c>
       <c r="AC42" t="inlineStr">
@@ -5210,24 +5210,24 @@
       </c>
       <c r="AD42" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>battery16</t>
+          <t>snrLast</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5251,7 +5251,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>store NA sentinel when E22 (UNSUPPORTED)</t>
+        </is>
+      </c>
       <c r="J43" t="inlineStr">
         <is>
           <t>N</t>
@@ -5261,66 +5265,54 @@
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Node_Operational</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr">
         <is>
-          <t>packet_sets_v0_1</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>link_metrics_v0; seq_ref_version_link_metrics_v0_1</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>i8</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>pct7+charging1+eta10m8</t>
+          <t>dB; 127 or -128 = NA/UNSUPPORTED</t>
         </is>
       </c>
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>TODO</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>on change + min_interval</t>
+          <t>on RX</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>periodic+threshold</t>
+          <t>event-driven</t>
         </is>
       </c>
       <c r="Z43" t="inlineStr"/>
       <c r="AA43" t="inlineStr"/>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>v0.1 packed container.</t>
+          <t>S03 required; E22 UNSUPPORTED -&gt; store NA sentinel (e.g. int8 127 or -128). Plumb through NodeTable and snapshots. seq_ref_version_link_metrics_v0_1.</t>
         </is>
       </c>
       <c r="AC43" t="inlineStr">
@@ -5330,14 +5322,14 @@
       </c>
       <c r="AD43" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>battery_pct7</t>
+          <t>battery16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5394,31 +5386,31 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>7 bits in battery16; 0-100</t>
-        </is>
-      </c>
-      <c r="T44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+          <t>pct7+charging1+eta10m8</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
@@ -5426,13 +5418,21 @@
           <t>C Tail-2</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr"/>
-      <c r="Y44" t="inlineStr"/>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
       <c r="Z44" t="inlineStr"/>
       <c r="AA44" t="inlineStr"/>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>Packed in battery16.</t>
+          <t>v0.1 packed container.</t>
         </is>
       </c>
       <c r="AC44" t="inlineStr">
@@ -5449,7 +5449,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>channel_throttle_step_u4</t>
+          <t>battery_pct7</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5515,14 +5515,22 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>4 bits in radio8</t>
-        </is>
-      </c>
-      <c r="T45" t="inlineStr"/>
-      <c r="U45" t="inlineStr"/>
+          <t>7 bits in battery16; 0-100</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
@@ -5536,7 +5544,7 @@
       <c r="AA45" t="inlineStr"/>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>Packed in radio8.</t>
+          <t>Packed in battery16.</t>
         </is>
       </c>
       <c r="AC45" t="inlineStr">
@@ -5546,14 +5554,14 @@
       </c>
       <c r="AD45" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>charging1</t>
+          <t>channel_throttle_step_u4</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5563,7 +5571,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5614,19 +5622,19 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>1 bit in battery16</t>
+          <t>4 bits in radio8</t>
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
@@ -5640,7 +5648,7 @@
       <c r="AA46" t="inlineStr"/>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>Packed in battery16.</t>
+          <t>Packed in radio8.</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5650,14 +5658,14 @@
       </c>
       <c r="AD46" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>eta10m8</t>
+          <t>charging1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5718,19 +5726,19 @@
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>8 bits in battery16; minutes to empty, 0=N/A</t>
+          <t>1 bit in battery16</t>
         </is>
       </c>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
@@ -5754,14 +5762,14 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>fix_type</t>
+          <t>eta10m8</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5771,7 +5779,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5810,7 +5818,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Node_Core_Tail</t>
+          <t>Node_Operational</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -5822,24 +5830,24 @@
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>bits in pos_quality16: no_fix/2d/3d/reserved</t>
+          <t>8 bits in battery16; minutes to empty, 0=N/A</t>
         </is>
       </c>
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X48" t="inlineStr"/>
@@ -5848,7 +5856,7 @@
       <c r="AA48" t="inlineStr"/>
       <c r="AB48" t="inlineStr">
         <is>
-          <t>Packed in pos_quality16.</t>
+          <t>Packed in battery16.</t>
         </is>
       </c>
       <c r="AC48" t="inlineStr">
@@ -5858,14 +5866,14 @@
       </c>
       <c r="AD48" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>pos_accuracy_bucket</t>
+          <t>fix_type</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5926,19 +5934,19 @@
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>bits in pos_quality16</t>
+          <t>bits in pos_quality16: no_fix/2d/3d/reserved</t>
         </is>
       </c>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W49" t="inlineStr">
@@ -5962,14 +5970,14 @@
       </c>
       <c r="AD49" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>pos_flags_small</t>
+          <t>pos_accuracy_bucket</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -6035,14 +6043,14 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>bits in pos_quality16; supersedes posFlags in v0.1</t>
+          <t>bits in pos_quality16</t>
         </is>
       </c>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="W50" t="inlineStr">
@@ -6056,7 +6064,7 @@
       <c r="AA50" t="inlineStr"/>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
+          <t>Packed in pos_quality16.</t>
         </is>
       </c>
       <c r="AC50" t="inlineStr">
@@ -6066,14 +6074,14 @@
       </c>
       <c r="AD50" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>pos_quality16</t>
+          <t>pos_flags_small</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -6130,31 +6138,23 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>packed: fix_type/sats/accuracy_bucket/pos_flags_small</t>
+          <t>bits in pos_quality16; supersedes posFlags in v0.1</t>
         </is>
       </c>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>5</t>
         </is>
       </c>
       <c r="W51" t="inlineStr">
@@ -6162,21 +6162,13 @@
           <t>B Tail-1</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y51" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr"/>
       <c r="Z51" t="inlineStr"/>
       <c r="AA51" t="inlineStr"/>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
+          <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
         </is>
       </c>
       <c r="AC51" t="inlineStr">
@@ -6193,7 +6185,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>radio8</t>
+          <t>pos_quality16</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6203,7 +6195,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6242,7 +6234,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>Node_Operational</t>
+          <t>Node_Core_Tail</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -6252,7 +6244,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -6262,33 +6254,41 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>txPower4+throttle4</t>
+          <t>packed: fix_type/sats/accuracy_bucket/pos_flags_small</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
       <c r="V52" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
-        </is>
-      </c>
-      <c r="X52" t="inlineStr"/>
-      <c r="Y52" t="inlineStr"/>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z52" t="inlineStr"/>
       <c r="AA52" t="inlineStr"/>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>v0.1 container.</t>
+          <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
         </is>
       </c>
       <c r="AC52" t="inlineStr">
@@ -6305,7 +6305,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>tx_power_step_u4</t>
+          <t>radio8</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6362,8 +6362,16 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R53" t="inlineStr">
         <is>
           <t>u8</t>
@@ -6371,14 +6379,14 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>4 bits in radio8</t>
+          <t>txPower4+throttle4</t>
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W53" t="inlineStr">
@@ -6392,7 +6400,7 @@
       <c r="AA53" t="inlineStr"/>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>Packed in radio8.</t>
+          <t>v0.1 container.</t>
         </is>
       </c>
       <c r="AC53" t="inlineStr">
@@ -6409,7 +6417,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>uptime10m_u8</t>
+          <t>tx_power_step_u4</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6419,7 +6427,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6466,16 +6474,8 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
           <t>u8</t>
@@ -6483,14 +6483,14 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>uptime in 10-minute units; masked-for-compare</t>
+          <t>4 bits in radio8</t>
         </is>
       </c>
       <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W54" t="inlineStr">
@@ -6498,21 +6498,13 @@
           <t>C Tail-2</t>
         </is>
       </c>
-      <c r="X54" t="inlineStr">
-        <is>
-          <t>on change + min_interval</t>
-        </is>
-      </c>
-      <c r="Y54" t="inlineStr">
-        <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
+      <c r="X54" t="inlineStr"/>
+      <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="inlineStr"/>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>v0.1; eligibility snapshot mask.</t>
+          <t>Packed in radio8.</t>
         </is>
       </c>
       <c r="AC54" t="inlineStr">
@@ -6529,17 +6521,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>node_name</t>
+          <t>uptime10m_u8</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6560,63 +6552,183 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>self-only in NVS (S03); not on-air in S03</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>identity_naming_persistence_eviction_v0_1</t>
-        </is>
-      </c>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S55" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>uptime in 10-minute units; masked-for-compare</t>
+        </is>
+      </c>
       <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr"/>
-      <c r="V55" t="inlineStr"/>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X55" t="inlineStr"/>
-      <c r="Y55" t="inlineStr"/>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
       <c r="Z55" t="inlineStr"/>
       <c r="AA55" t="inlineStr"/>
       <c r="AB55" t="inlineStr">
         <is>
+          <t>v0.1; eligibility snapshot mask.</t>
+        </is>
+      </c>
+      <c r="AC55" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>node_name</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>self-only in NVS (S03); not on-air in S03</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>identity_naming_persistence_eviction_v0_1</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr"/>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr"/>
+      <c r="Y56" t="inlineStr"/>
+      <c r="Z56" t="inlineStr"/>
+      <c r="AA56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr">
+        <is>
           <t>Human-readable name. S03: self set via BLE, persisted NVS; remote usually empty. Sxx: remote from over-air; authority rule: node-reported replaces local. UI: node_name -&gt; local phone name -&gt; short_id.</t>
         </is>
       </c>
-      <c r="AC55" t="inlineStr">
+      <c r="AC56" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="AD55" t="inlineStr">
+      <c r="AD56" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
@@ -6869,7 +6981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7091,58 +7203,70 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/seq_ref_version_link_metrics_v0_1.md</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
+          <t>S03 block: seq16/ref_core_seq16/last_applied_tail; last_payload_version_seen (debug); last_rx_rssi, snrLast (E22 NA); update rules.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
+          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
+          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
+          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>firmware/src/domain/node_table.cpp</t>
+          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>firmware/src/domain/node_table.cpp</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>firmware/src/domain/node_table.h</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>NodeEntry struct; NodeTable class; kRecordBytes=26.</t>
         </is>

</xml_diff>

<commit_message>
S03 WIP: seq/ref/version/link-metrics block (#377)
- Add seq_ref_version_link_metrics_v0_1.md: definitions (last_seq16,
  last_core_seq16, ref_core_seq16, last_applied_tail_ref_core_seq16),
  link metrics (last_rx_rssi, snrLast E22 NA sentinel), payloadVersion
  -> last_payload_version_seen (injected, debug only), update rules
- Master table: last_payload_version_seen (WIP, Injected); payloadVersion
  note; seq16/ref_core_seq16/last_applied_tail/last_rx_rssi/snrLast notes
  and seq_ref_version_link_metrics_v0_1 refs
- Regenerate XLSX + CSV; add SOURCES entry

Refs #351 #352. Follow-up: #375 (RSSI), #376 (snrLast sentinel).

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
+++ b/docs/product/wip/areas/nodetable/master_table/nodetable_master_table_v0_1.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD55"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -820,7 +820,7 @@
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Payload format version; first byte of payload.</t>
+          <t>On-air: first byte of payload. NodeTable/store may use last_payload_version_seen (injected, debug only). seq_ref_version_link_metrics_v0_1.</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -1220,7 +1220,7 @@
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Back-reference to Core sample seq16; distinct from seq16 in Common.</t>
+          <t>Tail-only ref. Back-reference to Core sample seq16. last_core_seq16 updates only on Core_Pos RX; tail apply only on Tail RX (seq_ref_version_link_metrics_v0_1).</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1364,7 +1364,7 @@
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>Dedupe key (nodeId48, seq16). last_seq in NodeEntry.</t>
+          <t>Dedupe key (nodeId48, seq16). last_seq in NodeEntry. Updates on any RX. last_core_seq16 updates only on Core_Pos RX; tail ref/apply only on Tail RX (seq_ref_version_link_metrics_v0_1).</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1877,17 +1877,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>snrLast</t>
+          <t>batteryPercent</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1897,23 +1897,27 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>battery_percent</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>TODO: add to NodeEntry/BLE if needed</t>
+          <t>in NodeEntry</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1925,71 +1929,91 @@
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>link_metrics_v0</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+          <t>tail2_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>dB</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
+          <t>0-100%; 0xFF=not present</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>7</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>on RX</t>
+          <t>on change + at forced Core</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>event-driven</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr"/>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>battery delta</t>
+        </is>
+      </c>
       <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>Not in current BLE record.</t>
-        </is>
-      </c>
+      <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>batteryPercent</t>
+          <t>sats</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1999,7 +2023,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2019,7 +2043,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>battery_percent</t>
+          <t>sats</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2046,12 +2070,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Node_Operational</t>
+          <t>Node_Core_Tail</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>tail2_packet_encoding_v0 §3.2</t>
+          <t>tail1_packet_encoding_v0 §3.2</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -2071,7 +2095,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>0-100%; 0xFF=not present</t>
+          <t>satellite count; 0=not present</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -2081,36 +2105,36 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>255</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
+          <t>B Tail-1</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>on change + at forced Core</t>
+          <t>Every Tail-1</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>battery delta</t>
-        </is>
-      </c>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>v0 canon. In v0.1 packed in pos_quality16; canonical field_key sats.</t>
+        </is>
+      </c>
       <c r="AC13" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -2125,7 +2149,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>uptimeSec</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2135,7 +2159,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2155,7 +2179,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>uptime_sec</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2182,17 +2206,17 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Node_Core_Tail</t>
+          <t>Node_Operational</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>tail1_packet_encoding_v0 §3.2</t>
+          <t>tail2_packet_encoding_v0 §3.2</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -2202,12 +2226,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u32</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>satellite count; 0=not present</t>
+          <t>seconds; 0xFFFFFFFF=not present</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -2217,12 +2241,12 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>4294967295</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>32</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -2232,19 +2256,19 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>Every Tail-1</t>
+          <t>on change + at forced Core</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>periodic</t>
+          <t>periodic+threshold</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>v0 canon. In v0.1 packed in pos_quality16; canonical field_key sats.</t>
+          <t>field_cadence: Tier B; packet is Node_Operational (0x04).</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
@@ -2261,17 +2285,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>uptimeSec</t>
+          <t>localAlias</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>LocalOnly</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2281,19 +2305,15 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>AppLocal</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>uptime_sec</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2301,7 +2321,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>in NodeEntry</t>
+          <t>app local storage</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2313,74 +2333,38 @@
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Node_Operational</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
-          <t>tail2_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>u32</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>seconds; 0xFFFFFFFF=not present</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>4294967295</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>on change + at forced Core</t>
-        </is>
-      </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>field_cadence: Tier B; packet is Node_Operational (0x04).</t>
+          <t>Local phone name; fallback when node_name (authoritative) empty. User-defined on phone; not over radio. Replaced by node-reported node_name when present (authority rule).</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -2390,42 +2374,46 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>localAlias</t>
+          <t>pos_age_s</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LocalOnly</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>CodeNow</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>AppLocal</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>pos_age_s</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2433,16 +2421,24 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>app local storage</t>
+          <t>BLE snapshot</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
           <t>N</t>
@@ -2451,23 +2447,39 @@
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>Tail-1 pos quality; not in Core</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>65535</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>B Tail-1</t>
         </is>
       </c>
       <c r="X16" t="inlineStr"/>
@@ -2476,7 +2488,7 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>Local phone name; fallback when node_name (authoritative) empty. User-defined on phone; not over radio. Replaced by node-reported node_name when present (authority rule).</t>
+          <t>S03 minimal. Age of last known position sample (independent from presence). Domain; not in BeaconCore payload (position_quality_v0).</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
@@ -2486,14 +2498,14 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>pos_age_s</t>
+          <t>pos_valid</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2523,7 +2535,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>pos_age_s</t>
+          <t>pos_valid</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2533,7 +2545,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>BLE snapshot (flags bit1)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2543,12 +2555,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2557,41 +2569,29 @@
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Tail-1 pos quality; not in Core</t>
-        </is>
-      </c>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>seconds</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>65535</t>
-        </is>
-      </c>
+          <t>flags bit 0x02; Core implies valid</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
+          <t>A Core</t>
         </is>
       </c>
       <c r="X17" t="inlineStr"/>
@@ -2600,7 +2600,7 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>S03 minimal. Age of last known position sample (independent from presence). Domain; not in BeaconCore payload (position_quality_v0).</t>
+          <t>Domain/BLE only; not on-air in BeaconCore (Core only when fix valid).</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2617,17 +2617,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>pos_valid</t>
+          <t>is_stale</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2637,27 +2637,23 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>pos_valid</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>BLE snapshot (flags bit1)</t>
+          <t>computed at export</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2681,7 +2677,11 @@
         </is>
       </c>
       <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>presence_and_age_semantics_v0_1</t>
+        </is>
+      </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>flags bit 0x02; Core implies valid</t>
+          <t>flags bit 0x04; last_seen_age_s &gt; expected_interval_s + grace_s</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -2703,7 +2703,7 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>A Core</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X18" t="inlineStr"/>
@@ -2712,7 +2712,7 @@
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>Domain/BLE only; not on-air in BeaconCore (Core only when fix valid).</t>
+          <t>S03 minimal. expected_interval_s = max_silence_10s * 10; grace_s hysteresis TBD. Self: TX heartbeat updates last_seen_ms so self does not appear stale (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
@@ -2722,14 +2722,14 @@
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>is_stale</t>
+          <t>last_seen_age_s</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>computed at export</t>
+          <t>computed at export from last_seen_ms</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2775,12 +2775,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2789,30 +2789,22 @@
         </is>
       </c>
       <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>presence_and_age_semantics_v0_1</t>
-        </is>
-      </c>
+      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>flags bit 0x04; last_seen_age_s &gt; expected_interval_s + grace_s</t>
+          <t>(now_ms - last_seen_ms)/1000</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -2824,7 +2816,7 @@
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>S03 minimal. expected_interval_s = max_silence_10s * 10; grace_s hysteresis TBD. Self: TX heartbeat updates last_seen_ms so self does not appear stale (presence_and_age_semantics_v0_1).</t>
+          <t>S03 minimal. floor((now_ms - last_seen_ms)/1000) at export; BLE convenience; derived from last_seen_ms. See presence_and_age_semantics_v0_1.</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -2841,17 +2833,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>last_seen_age_s</t>
+          <t>in_use</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>LocalOnly</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2861,15 +2853,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>AppLocal</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>in_use</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>N</t>
@@ -2877,24 +2873,16 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>computed at export from last_seen_ms</t>
+          <t>internal slot only</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>N</t>
@@ -2906,14 +2894,10 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>u16</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>(now_ms - last_seen_ms)/1000</t>
-        </is>
-      </c>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
@@ -2928,7 +2912,7 @@
       <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>S03 minimal. floor((now_ms - last_seen_ms)/1000) at export; BLE convenience; derived from last_seen_ms. See presence_and_age_semantics_v0_1.</t>
+          <t>Internal; not in BLE.</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -2945,7 +2929,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>in_use</t>
+          <t>is_self</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2975,26 +2959,34 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>in_use</t>
+          <t>is_self</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>internal slot only</t>
+          <t>BLE snapshot (flags bit0)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>N</t>
@@ -3009,10 +3001,18 @@
           <t>bool</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>flags bit 0x01</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W21" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3022,11 +3022,7 @@
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr"/>
-      <c r="AB21" t="inlineStr">
-        <is>
-          <t>Internal; not in BLE.</t>
-        </is>
-      </c>
+      <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3034,14 +3030,14 @@
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>is_self</t>
+          <t>last_applied_tail_ref_core_seq16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3051,7 +3047,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LocalOnly</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3061,7 +3057,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AppLocal</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3071,60 +3067,44 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>is_self</t>
+          <t>last_applied_tail_ref_core_seq16</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>BLE snapshot (flags bit0)</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>tail1_packet_encoding_v0; at most one Tail per Core</t>
+        </is>
+      </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>flags bit 0x01</t>
-        </is>
-      </c>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3134,7 +3114,11 @@
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>Variant 2: dedupe second Tail-1 for same ref_core_seq16. Updates only on Tail RX when applied (seq_ref_version_link_metrics_v0_1).</t>
+        </is>
+      </c>
       <c r="AC22" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3142,14 +3126,14 @@
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>last_applied_tail_ref_core_seq16</t>
+          <t>short_id</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3159,7 +3143,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3169,7 +3153,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3179,33 +3163,41 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>last_applied_tail_ref_core_seq16</t>
+          <t>short_id</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>BLE snapshot</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>tail1_packet_encoding_v0; at most one Tail per Core</t>
-        </is>
-      </c>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
@@ -3213,10 +3205,18 @@
           <t>u16</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>CRC16-CCITT over node_id LE</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="W23" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3228,7 +3228,7 @@
       <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>Variant 2: dedupe second Tail-1 for same ref_core_seq16.</t>
+          <t>Display only; not protocol key. Reserved 0x0000/0xFFFF handled.</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
@@ -3245,7 +3245,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>short_id</t>
+          <t>short_id_collision</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>short_id</t>
+          <t>short_id_collision</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>BLE snapshot (flags bit3)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -3295,12 +3295,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3314,19 +3314,19 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>CRC16-CCITT over node_id LE</t>
+          <t>flags bit 0x08</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
@@ -3338,11 +3338,7 @@
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr">
-        <is>
-          <t>Display only; not protocol key. Reserved 0x0000/0xFFFF handled.</t>
-        </is>
-      </c>
+      <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3357,17 +3353,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>short_id_collision</t>
+          <t>last_rx_rssi</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3377,7 +3373,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3387,7 +3383,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>short_id_collision</t>
+          <t>last_rx_rssi</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3397,7 +3393,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>BLE snapshot (flags bit3)</t>
+          <t>BLE snapshot</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -3407,7 +3403,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>23</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -3421,24 +3417,28 @@
         </is>
       </c>
       <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>link_metrics_v0</t>
+        </is>
+      </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>i8</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>flags bit 0x08</t>
+          <t>dBm</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
@@ -3446,11 +3446,23 @@
           <t>Derived/Injected</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>on RX</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>event-driven</t>
+        </is>
+      </c>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>S03 required. rssiLast; updated on any RX from that node. Units raw or dBm TBD. seq_ref_version_link_metrics_v0_1.</t>
+        </is>
+      </c>
       <c r="AC25" t="inlineStr">
         <is>
           <t>Implemented</t>
@@ -3458,14 +3470,14 @@
       </c>
       <c r="AD25" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>last_rx_rssi</t>
+          <t>last_seen_ms</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3475,7 +3487,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3495,7 +3507,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>last_rx_rssi</t>
+          <t>last_seen_ms</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3505,54 +3517,38 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>BLE snapshot</t>
+          <t>internal; BLE exports last_seen_age_s derived</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>link_metrics_v0</t>
-        </is>
-      </c>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>i8</t>
+          <t>u32</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>dBm</t>
+          <t>uptime ms</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -3572,7 +3568,7 @@
       <c r="AA26" t="inlineStr"/>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>rssiLast; receiver-side only.</t>
+          <t>Exported as lastSeenAgeS (age_s) in BLE.</t>
         </is>
       </c>
       <c r="AC26" t="inlineStr">
@@ -3589,49 +3585,41 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>last_seen_ms</t>
+          <t>networkName</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CodeNow</t>
+          <t>Idea</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>last_seen_ms</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>internal; BLE exports last_seen_age_s derived</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>N</t>
@@ -3645,79 +3633,67 @@
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>index §4</t>
+        </is>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>u32</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>uptime ms</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>on RX</t>
-        </is>
-      </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>event-driven</t>
-        </is>
-      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="inlineStr"/>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>Exported as lastSeenAgeS (age_s) in BLE.</t>
+          <t>Out-of-scope S03; NOT sent in v0 beacon; future session-join.</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>networkName</t>
+          <t>hops</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Routing/Mesh</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Mesh_future</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3747,28 +3723,36 @@
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
-          <t>index §4</t>
+          <t>meshtastic-nodetable.md §3</t>
         </is>
       </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>hops_away</t>
+        </is>
+      </c>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr"/>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>Out-of-scope S03; NOT sent in v0 beacon; future session-join.</t>
+          <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
       <c r="AC28" t="inlineStr">
@@ -3778,14 +3762,14 @@
       </c>
       <c r="AD28" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>hops</t>
+          <t>last_direct_time</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3795,7 +3779,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Routing/Mesh</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3835,21 +3819,17 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
-          <t>meshtastic-nodetable.md §3</t>
+          <t>naviga_mesh_protocol_concept_v1_4.md</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>u8</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>hops_away</t>
-        </is>
-      </c>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="inlineStr"/>
@@ -3864,7 +3844,7 @@
       <c r="AA29" t="inlineStr"/>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>No mesh routing in Naviga v0.</t>
+          <t>Time of last direct RX from this node; mesh concept. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC29" t="inlineStr">
@@ -3874,14 +3854,14 @@
       </c>
       <c r="AD29" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>last_direct_time</t>
+          <t>next_hop</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3891,7 +3871,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Routing/Mesh</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3931,17 +3911,21 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr">
         <is>
-          <t>naviga_mesh_protocol_concept_v1_4.md</t>
+          <t>meshtastic-nodetable.md §3</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>last byte of node num</t>
+        </is>
+      </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr"/>
@@ -3956,7 +3940,7 @@
       <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>Time of last direct RX from this node; mesh concept. Non-goal v0.</t>
+          <t>No mesh routing in Naviga v0.</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr">
@@ -3966,14 +3950,14 @@
       </c>
       <c r="AD30" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>next_hop</t>
+          <t>pos_history</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3983,7 +3967,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Routing/Mesh</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3993,7 +3977,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4023,19 +4007,19 @@
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr">
         <is>
-          <t>meshtastic-nodetable.md §3</t>
+          <t>naviga_mesh_protocol_concept_v1_4.md</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>array</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>last byte of node num</t>
+          <t>short history of positions</t>
         </is>
       </c>
       <c r="T31" t="inlineStr"/>
@@ -4052,7 +4036,7 @@
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>No mesh routing in Naviga v0.</t>
+          <t>Optional pos_history_X; mesh concept. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -4062,14 +4046,14 @@
       </c>
       <c r="AD31" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>pos_history</t>
+          <t>role_params</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4079,7 +4063,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4126,12 +4110,12 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>enum/params</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>short history of positions</t>
+          <t>role_pos_update_interval_X etc</t>
         </is>
       </c>
       <c r="T32" t="inlineStr"/>
@@ -4148,7 +4132,7 @@
       <c r="AA32" t="inlineStr"/>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>Optional pos_history_X; mesh concept. Non-goal v0.</t>
+          <t>Role-based delivery params; mesh concept. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -4158,14 +4142,14 @@
       </c>
       <c r="AD32" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>role_params</t>
+          <t>rssi_direct</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4175,7 +4159,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4185,7 +4169,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4215,21 +4199,17 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>naviga_mesh_protocol_concept_v1_4.md</t>
+          <t>meshtastic research</t>
         </is>
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>enum/params</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>role_pos_update_interval_X etc</t>
-        </is>
-      </c>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr"/>
@@ -4244,7 +4224,7 @@
       <c r="AA33" t="inlineStr"/>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>Role-based delivery params; mesh concept. Non-goal v0.</t>
+          <t>Direct-link RSSI; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC33" t="inlineStr">
@@ -4254,14 +4234,14 @@
       </c>
       <c r="AD33" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>rssi_direct</t>
+          <t>snr_direct</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4336,7 +4316,7 @@
       <c r="AA34" t="inlineStr"/>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>Direct-link RSSI; Mesh_future. Non-goal v0.</t>
+          <t>Direct-link SNR; Mesh_future. Non-goal v0.</t>
         </is>
       </c>
       <c r="AC34" t="inlineStr">
@@ -4353,27 +4333,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>snr_direct</t>
+          <t>is_grey</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mesh_future</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ReceiverInjected</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4390,33 +4370,45 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>meshtastic research</t>
-        </is>
-      </c>
+      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr"/>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>same as is_stale (flags bit 0x04)</t>
+        </is>
+      </c>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="W35" t="inlineStr">
         <is>
           <t>Derived/Injected</t>
@@ -4428,34 +4420,34 @@
       <c r="AA35" t="inlineStr"/>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>Direct-link SNR; Mesh_future. Non-goal v0.</t>
+          <t>Alias; superseded-by is_stale (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC35" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="AD35" t="inlineStr">
         <is>
-          <t>Injected</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>is_grey</t>
+          <t>posFlags</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4465,74 +4457,106 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>pos_flags</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>in NodeEntry</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Node_Core_Tail</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>tail1_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>same as is_stale (flags bit 0x04)</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
+          <t>bit0=position valid; 1-7 reserved</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X36" t="inlineStr"/>
-      <c r="Y36" t="inlineStr"/>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z36" t="inlineStr"/>
       <c r="AA36" t="inlineStr"/>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>Alias; superseded-by is_stale (presence_and_age_semantics_v0_1).</t>
+          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
         </is>
       </c>
       <c r="AC36" t="inlineStr">
@@ -4542,14 +4566,14 @@
       </c>
       <c r="AD36" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>posFlags</t>
+          <t>pos_sats</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4574,24 +4598,16 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>pos_flags</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>in NodeEntry</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>N</t>
@@ -4601,29 +4617,17 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Node_Core_Tail</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr">
         <is>
-          <t>tail1_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
           <t>u8</t>
@@ -4631,76 +4635,56 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>bit0=position valid; 1-7 reserved</t>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="V37" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+          <t>alias for sats</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr">
         <is>
           <t>B Tail-1</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y37" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="inlineStr"/>
       <c r="AA37" t="inlineStr"/>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>v0 canon. Superseded by pos_flags_small (v0.1 packed in pos_quality16).</t>
+          <t>Alias; superseded-by sats.</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD37" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>pos_sats</t>
+          <t>aliveStatus</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Superseded</t>
+          <t>WIP</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4732,14 +4716,26 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Alive</t>
+        </is>
+      </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>packet_sets_v0_1</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
+          <t>alive_packet_encoding_v0 §3.2</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R38" t="inlineStr">
         <is>
           <t>u8</t>
@@ -4747,51 +4743,63 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>alias for sats</t>
+          <t>0x00=alive_no_fix</t>
         </is>
       </c>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
-        </is>
-      </c>
-      <c r="X38" t="inlineStr"/>
-      <c r="Y38" t="inlineStr"/>
+          <t>A Core</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>no-fix liveness</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z38" t="inlineStr"/>
       <c r="AA38" t="inlineStr"/>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>Alias; superseded-by sats.</t>
+          <t>Not promoted to S03; unused/stubbed. Covered by minimal model (presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Stubbed</t>
         </is>
       </c>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>aliveStatus</t>
+          <t>PositionQuality</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4801,7 +4809,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4828,80 +4836,56 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Alive</t>
-        </is>
-      </c>
+      <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr">
         <is>
-          <t>alive_packet_encoding_v0 §3.2</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>position_quality_v0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>0x00=alive_no_fix</t>
+          <t>Core + Tail-1 posFlags/sats + age</t>
         </is>
       </c>
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+      <c r="V39" t="inlineStr"/>
       <c r="W39" t="inlineStr">
         <is>
-          <t>A Core</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>no-fix liveness</t>
-        </is>
-      </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>Not promoted to S03; unused/stubbed. Covered by minimal model (presence_and_age_semantics_v0_1).</t>
+          <t>Not promoted to S03; policy-only derived. Covered by minimal model (pos_age_s, posFlags/sats; presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>Stubbed</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="AD39" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PositionQuality</t>
+          <t>activityState</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4911,7 +4895,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Activity</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4951,19 +4935,19 @@
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
-          <t>position_quality_v0</t>
+          <t>activity_state_v0</t>
         </is>
       </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Core + Tail-1 posFlags/sats + age</t>
+          <t>Unknown/Active/Stale/Lost</t>
         </is>
       </c>
       <c r="T40" t="inlineStr"/>
@@ -4974,13 +4958,21 @@
           <t>Derived/Injected</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr"/>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>derived on RX</t>
+        </is>
+      </c>
       <c r="Y40" t="inlineStr"/>
-      <c r="Z40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>T_active, T_stale params</t>
+        </is>
+      </c>
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>Not promoted to S03; policy-only derived. Covered by minimal model (pos_age_s, posFlags/sats; presence_and_age_semantics_v0_1).</t>
+          <t>Not promoted to S03; policy-only derived. Covered by minimal model (is_stale, last_seen_age_s; presence_and_age_semantics_v0_1).</t>
         </is>
       </c>
       <c r="AC40" t="inlineStr">
@@ -4997,17 +4989,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>activityState</t>
+          <t>role_id</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Informative</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5017,7 +5009,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>NodeOwned</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -5041,50 +5033,62 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Node_Informative</t>
+        </is>
+      </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>activity_state_v0</t>
+          <t>packet_sets_v0_1</t>
         </is>
       </c>
       <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Unknown/Active/Stale/Lost</t>
+          <t>role identifier</t>
         </is>
       </c>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>derived on RX</t>
-        </is>
-      </c>
-      <c r="Y41" t="inlineStr"/>
-      <c r="Z41" t="inlineStr">
-        <is>
-          <t>T_active, T_stale params</t>
-        </is>
-      </c>
+          <t>periodic + changed-boost</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr"/>
       <c r="AA41" t="inlineStr"/>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>Not promoted to S03; policy-only derived. Covered by minimal model (is_stale, last_seen_age_s; presence_and_age_semantics_v0_1).</t>
+          <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
         </is>
       </c>
       <c r="AC41" t="inlineStr">
@@ -5094,19 +5098,19 @@
       </c>
       <c r="AD41" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>Config</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>role_id</t>
+          <t>last_payload_version_seen</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Informative</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5121,7 +5125,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5135,7 +5139,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>debug only; not persisted</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr">
         <is>
           <t>N</t>
@@ -5145,25 +5153,17 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Node_Informative</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr">
         <is>
-          <t>packet_sets_v0_1</t>
+          <t>seq_ref_version_link_metrics_v0_1</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>u8</t>
@@ -5171,36 +5171,36 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>role identifier</t>
+          <t>last seen payloadVersion byte</t>
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>periodic + changed-boost</t>
+          <t>on RX</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>periodic</t>
+          <t>event-driven</t>
         </is>
       </c>
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>v0.1 new; Informative. CONFLICT: hw/fw remain u16 in canon.</t>
+          <t>Injected; decoder/debug aid only. Not user-facing; not persisted. Optional in NodeEntry. seq_ref_version_link_metrics_v0_1.</t>
         </is>
       </c>
       <c r="AC42" t="inlineStr">
@@ -5210,24 +5210,24 @@
       </c>
       <c r="AD42" t="inlineStr">
         <is>
-          <t>Config</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>battery16</t>
+          <t>snrLast</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Injected</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>NodeOwned</t>
+          <t>ReceiverInjected</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5251,7 +5251,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>store NA sentinel when E22 (UNSUPPORTED)</t>
+        </is>
+      </c>
       <c r="J43" t="inlineStr">
         <is>
           <t>N</t>
@@ -5261,66 +5265,54 @@
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Node_Operational</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr">
         <is>
-          <t>packet_sets_v0_1</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+          <t>link_metrics_v0; seq_ref_version_link_metrics_v0_1</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>i8</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>pct7+charging1+eta10m8</t>
+          <t>dB; 127 or -128 = NA/UNSUPPORTED</t>
         </is>
       </c>
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>TODO</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
+          <t>Derived/Injected</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>on change + min_interval</t>
+          <t>on RX</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>periodic+threshold</t>
+          <t>event-driven</t>
         </is>
       </c>
       <c r="Z43" t="inlineStr"/>
       <c r="AA43" t="inlineStr"/>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>v0.1 packed container.</t>
+          <t>S03 required; E22 UNSUPPORTED -&gt; store NA sentinel (e.g. int8 127 or -128). Plumb through NodeTable and snapshots. seq_ref_version_link_metrics_v0_1.</t>
         </is>
       </c>
       <c r="AC43" t="inlineStr">
@@ -5330,14 +5322,14 @@
       </c>
       <c r="AD43" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Injected</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>battery_pct7</t>
+          <t>battery16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5394,31 +5386,31 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>7 bits in battery16; 0-100</t>
-        </is>
-      </c>
-      <c r="T44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+          <t>pct7+charging1+eta10m8</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
       <c r="V44" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
@@ -5426,13 +5418,21 @@
           <t>C Tail-2</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr"/>
-      <c r="Y44" t="inlineStr"/>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
       <c r="Z44" t="inlineStr"/>
       <c r="AA44" t="inlineStr"/>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>Packed in battery16.</t>
+          <t>v0.1 packed container.</t>
         </is>
       </c>
       <c r="AC44" t="inlineStr">
@@ -5449,7 +5449,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>channel_throttle_step_u4</t>
+          <t>battery_pct7</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5515,14 +5515,22 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>4 bits in radio8</t>
-        </is>
-      </c>
-      <c r="T45" t="inlineStr"/>
-      <c r="U45" t="inlineStr"/>
+          <t>7 bits in battery16; 0-100</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
@@ -5536,7 +5544,7 @@
       <c r="AA45" t="inlineStr"/>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>Packed in radio8.</t>
+          <t>Packed in battery16.</t>
         </is>
       </c>
       <c r="AC45" t="inlineStr">
@@ -5546,14 +5554,14 @@
       </c>
       <c r="AD45" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>charging1</t>
+          <t>channel_throttle_step_u4</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5563,7 +5571,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5614,19 +5622,19 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>1 bit in battery16</t>
+          <t>4 bits in radio8</t>
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W46" t="inlineStr">
@@ -5640,7 +5648,7 @@
       <c r="AA46" t="inlineStr"/>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>Packed in battery16.</t>
+          <t>Packed in radio8.</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5650,14 +5658,14 @@
       </c>
       <c r="AD46" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>eta10m8</t>
+          <t>charging1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5718,19 +5726,19 @@
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>8 bits in battery16; minutes to empty, 0=N/A</t>
+          <t>1 bit in battery16</t>
         </is>
       </c>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W47" t="inlineStr">
@@ -5754,14 +5762,14 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>fix_type</t>
+          <t>eta10m8</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5771,7 +5779,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5810,7 +5818,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Node_Core_Tail</t>
+          <t>Node_Operational</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -5822,24 +5830,24 @@
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>bits in pos_quality16: no_fix/2d/3d/reserved</t>
+          <t>8 bits in battery16; minutes to empty, 0=N/A</t>
         </is>
       </c>
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>B Tail-1</t>
+          <t>C Tail-2</t>
         </is>
       </c>
       <c r="X48" t="inlineStr"/>
@@ -5848,7 +5856,7 @@
       <c r="AA48" t="inlineStr"/>
       <c r="AB48" t="inlineStr">
         <is>
-          <t>Packed in pos_quality16.</t>
+          <t>Packed in battery16.</t>
         </is>
       </c>
       <c r="AC48" t="inlineStr">
@@ -5858,14 +5866,14 @@
       </c>
       <c r="AD48" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>pos_accuracy_bucket</t>
+          <t>fix_type</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5926,19 +5934,19 @@
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>bits in pos_quality16</t>
+          <t>bits in pos_quality16: no_fix/2d/3d/reserved</t>
         </is>
       </c>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W49" t="inlineStr">
@@ -5962,14 +5970,14 @@
       </c>
       <c r="AD49" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>HW</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>pos_flags_small</t>
+          <t>pos_accuracy_bucket</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -6035,14 +6043,14 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>bits in pos_quality16; supersedes posFlags in v0.1</t>
+          <t>bits in pos_quality16</t>
         </is>
       </c>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="W50" t="inlineStr">
@@ -6056,7 +6064,7 @@
       <c r="AA50" t="inlineStr"/>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
+          <t>Packed in pos_quality16.</t>
         </is>
       </c>
       <c r="AC50" t="inlineStr">
@@ -6066,14 +6074,14 @@
       </c>
       <c r="AD50" t="inlineStr">
         <is>
-          <t>HW</t>
+          <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>pos_quality16</t>
+          <t>pos_flags_small</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -6130,31 +6138,23 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>u8</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>packed: fix_type/sats/accuracy_bucket/pos_flags_small</t>
+          <t>bits in pos_quality16; supersedes posFlags in v0.1</t>
         </is>
       </c>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>5</t>
         </is>
       </c>
       <c r="W51" t="inlineStr">
@@ -6162,21 +6162,13 @@
           <t>B Tail-1</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr">
-        <is>
-          <t>Every Tail-1</t>
-        </is>
-      </c>
-      <c r="Y51" t="inlineStr">
-        <is>
-          <t>periodic</t>
-        </is>
-      </c>
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr"/>
       <c r="Z51" t="inlineStr"/>
       <c r="AA51" t="inlineStr"/>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
+          <t>Mapping from v0 posFlags; packed in pos_quality16.</t>
         </is>
       </c>
       <c r="AC51" t="inlineStr">
@@ -6193,7 +6185,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>radio8</t>
+          <t>pos_quality16</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6203,7 +6195,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>RadioContext</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6242,7 +6234,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>Node_Operational</t>
+          <t>Node_Core_Tail</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -6252,7 +6244,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -6262,33 +6254,41 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>u8</t>
+          <t>u16</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>txPower4+throttle4</t>
+          <t>packed: fix_type/sats/accuracy_bucket/pos_flags_small</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
       <c r="V52" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>16</t>
         </is>
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>C Tail-2</t>
-        </is>
-      </c>
-      <c r="X52" t="inlineStr"/>
-      <c r="Y52" t="inlineStr"/>
+          <t>B Tail-1</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>Every Tail-1</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
       <c r="Z52" t="inlineStr"/>
       <c r="AA52" t="inlineStr"/>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>v0.1 container.</t>
+          <t>v0.1 container; replaces separate posFlags(1)+sats(1) in v0.</t>
         </is>
       </c>
       <c r="AC52" t="inlineStr">
@@ -6305,7 +6305,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>tx_power_step_u4</t>
+          <t>radio8</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6362,8 +6362,16 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R53" t="inlineStr">
         <is>
           <t>u8</t>
@@ -6371,14 +6379,14 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>4 bits in radio8</t>
+          <t>txPower4+throttle4</t>
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W53" t="inlineStr">
@@ -6392,7 +6400,7 @@
       <c r="AA53" t="inlineStr"/>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>Packed in radio8.</t>
+          <t>v0.1 container.</t>
         </is>
       </c>
       <c r="AC53" t="inlineStr">
@@ -6409,7 +6417,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>uptime10m_u8</t>
+          <t>tx_power_step_u4</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6419,7 +6427,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Telemetry/Health</t>
+          <t>RadioContext</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6466,16 +6474,8 @@
           <t>packet_sets_v0_1</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>OPT</t>
-        </is>
-      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
           <t>u8</t>
@@ -6483,14 +6483,14 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>uptime in 10-minute units; masked-for-compare</t>
+          <t>4 bits in radio8</t>
         </is>
       </c>
       <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W54" t="inlineStr">
@@ -6498,21 +6498,13 @@
           <t>C Tail-2</t>
         </is>
       </c>
-      <c r="X54" t="inlineStr">
-        <is>
-          <t>on change + min_interval</t>
-        </is>
-      </c>
-      <c r="Y54" t="inlineStr">
-        <is>
-          <t>periodic+threshold</t>
-        </is>
-      </c>
+      <c r="X54" t="inlineStr"/>
+      <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="inlineStr"/>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>v0.1; eligibility snapshot mask.</t>
+          <t>Packed in radio8.</t>
         </is>
       </c>
       <c r="AC54" t="inlineStr">
@@ -6529,17 +6521,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>node_name</t>
+          <t>uptime10m_u8</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Telemetry/Health</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6560,63 +6552,183 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>self-only in NVS (S03); not on-air in S03</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Node_Operational</t>
+        </is>
+      </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>identity_naming_persistence_eviction_v0_1</t>
-        </is>
-      </c>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
+          <t>packet_sets_v0_1</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>OPT</t>
+        </is>
+      </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="S55" t="inlineStr"/>
+          <t>u8</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>uptime in 10-minute units; masked-for-compare</t>
+        </is>
+      </c>
       <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr"/>
-      <c r="V55" t="inlineStr"/>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>Derived/Injected</t>
-        </is>
-      </c>
-      <c r="X55" t="inlineStr"/>
-      <c r="Y55" t="inlineStr"/>
+          <t>C Tail-2</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>on change + min_interval</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>periodic+threshold</t>
+        </is>
+      </c>
       <c r="Z55" t="inlineStr"/>
       <c r="AA55" t="inlineStr"/>
       <c r="AB55" t="inlineStr">
         <is>
+          <t>v0.1; eligibility snapshot mask.</t>
+        </is>
+      </c>
+      <c r="AC55" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>node_name</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>NodeOwned</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>self-only in NVS (S03); not on-air in S03</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>identity_naming_persistence_eviction_v0_1</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr"/>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>Derived/Injected</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr"/>
+      <c r="Y56" t="inlineStr"/>
+      <c r="Z56" t="inlineStr"/>
+      <c r="AA56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr">
+        <is>
           <t>Human-readable name. S03: self set via BLE, persisted NVS; remote usually empty. Sxx: remote from over-air; authority rule: node-reported replaces local. UI: node_name -&gt; local phone name -&gt; short_id.</t>
         </is>
       </c>
-      <c r="AC55" t="inlineStr">
+      <c r="AC56" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="AD55" t="inlineStr">
+      <c r="AD56" t="inlineStr">
         <is>
           <t>Config</t>
         </is>
@@ -6869,7 +6981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7091,58 +7203,70 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/seq_ref_version_link_metrics_v0_1.md</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
+          <t>S03 block: seq16/ref_core_seq16/last_applied_tail; last_payload_version_seen (debug); last_rx_rssi, snrLast (E22 NA); update rules.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
+          <t>docs/product/wip/areas/nodetable/policy/tx_priority_and_arbitration_v0_1.md</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
+          <t>TX priority P0-P3; coalesce_key; hybrid expired_counter (WIP).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
+          <t>docs/product/wip/areas/nodetable/research/meshastic-nodetable.md</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
+          <t>Meshtastic NodeDB categories; transferability; hops_away, next_hop, last_heard.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>firmware/src/domain/node_table.cpp</t>
+          <t>docs/product/wip/areas/nodetable/research/naviga-current-state.md</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+          <t>BLE 26-byte record layout; NodeRecordV1; write/read paths.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>firmware/src/domain/node_table.cpp</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>get_page/get_snapshot_page BLE layout; upsert_remote; apply_tail1/tail2/info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>firmware/src/domain/node_table.h</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>NodeEntry struct; NodeTable class; kRecordBytes=26.</t>
         </is>

</xml_diff>